<commit_message>
feat: filter non-faculty positions, parse real institutions, and add research topics column
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -461,25 +461,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="53" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="210" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="67" customWidth="1" min="3" max="3"/>
+    <col width="77" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -500,65 +501,70 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Research Topics</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Tenure Track</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Salary</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Summary (Gemini)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Date Added</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Last Verified</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
@@ -567,59 +573,59 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Civil, Construction and Environmental Engineering -TransportationEngineering -AssistantProfessor</t>
+          <t>Assistant Professor of Transportation Engineering</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering</t>
+          <t>University of Alabama</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering</t>
+          <t>Department of Civil, Construction and Environmental Engineering</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Transportation Engineering, Civil Engineering, Transportation Systems</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor University of Alabama Civil, Construction and Environmental Engineering Tuscaloosa, Alabama United States Date Posted Nov. 3, 2025 Deadline Open until filled Position Starts Aug. 16, 2026</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Review begins immediately / Open</t>
+          <t>Tuscaloosa, AL</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Civil, Construction and Environmental Engineering - Transportation Engineering - Assistant Professor University of Alabama Civil, Construction and Environmental Engineering Tuscaloosa, Alabama United ...</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>The Department of Civil, Construction and Environmental Engineering at the University of Alabama is hiring a tenure-track Assistant Professor in Transportation Engineering, requiring an earned doctorate in civil engineering or a closely related field. | Research Topics: Transportation Engineering, Civil Engineering, Transportation Systems</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>https://engineering.academickeys.com/job/s9z6epb3/Civil-Construction-and-Environmental-Engineering--Transportation-Engineering--Assistant-Professor</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
@@ -627,16 +633,21 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
-        <v>39.0691039</v>
-      </c>
       <c r="O2" s="2" t="n">
-        <v>-108.5607374</v>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
+        <v>33.2120822</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>-87.53967350000001</v>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>daabd65ea8fe188a</t>
         </is>
@@ -645,59 +656,59 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Postdoctoral Scholar</t>
+          <t>Assistant Professor of Transportation Engineering</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>AcademicKeys Listed Institution</t>
+          <t>South Dakota State University</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering</t>
+          <t>Civil and Environmental Engineering</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Transportation Engineering, Civil Infrastructure, Traffic Engineering</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Review begins immediately / Open</t>
+          <t>Brookings, SD</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Postdoctoral Scholar Michigan Technological University Civil, Environmental, and Geospatial Engineering Houghton, Michigan United States Date Posted Jul. 13, 2026 Deadline Aug. 1, 2026 Position Starts...</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/7yb6uoel/Postdoctoral-Scholar</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>South Dakota State University invites applications for a tenure-track Assistant Professor of Transportation Engineering in the Department of Civil and Environmental Engineering, requiring a Ph.D. in Civil Engineering or a closely related field. | Research Topics: Transportation Engineering, Civil Infrastructure, Traffic Engineering</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>https://engineering.academickeys.com/job/m4lk5asr/Assistant-Professor-of-Transportation-Engineering</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
@@ -705,73 +716,82 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>aa223cc351175091</t>
+      <c r="O3" s="2" t="n">
+        <v>44.344449</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>-96.79823709999999</v>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>9b7d5de4753a514b</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AssistantProfessorofTransportationEngineering</t>
+          <t>Assistant/Associate Professor of Civil Engineering (Transportation)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>AcademicKeys Listed Institution</t>
+          <t>Trine University</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering</t>
+          <t>Allen School of Engineering &amp; Computing</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>Transportation Engineering, Civil Infrastructure, Traffic Systems</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>Unspecified</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Review begins immediately / Open</t>
+          <t>Angola, IN</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Assistant Professor of Transportation Engineering South Dakota State University Civil and Environmental Engineering Brookings, South Dakota United States Date Posted Jul. 2, 2026 Deadline Aug. 16, 202...</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/m4lk5asr/Assistant-Professor-of-Transportation-Engineering</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Trine University invites applications for an Assistant or Associate Professor of Civil Engineering specializing in transportation, requiring a Ph.D. in Civil Engineering or a closely related field. | Research Topics: Transportation Engineering, Civil Infrastructure, Traffic Systems</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>https://engineering.academickeys.com/job/e8akh47s/AssistantAssociate-Professor--Civil-Engineering-Transportation</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
@@ -779,73 +799,78 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>9b7d5de4753a514b</t>
+      <c r="O4" s="2" t="n">
+        <v>41.6311141</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>-85.0105982</v>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>87a4115bef0ef2e7</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Research Fellow (TransportationEngineering)</t>
+          <t>Civil, Construction and Environmental Engineering - Assistant Professor</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>AcademicKeys Listed Institution</t>
+          <t>University of Alabama</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+          <t>Transportation / Civil Engineering</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Unspecified</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Review begins immediately / Open</t>
+          <t>Tuscaloosa, Alabama</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Research Fellow ( Transportation Engineering) Nanyang Technological University School of Civil and Environmental Engineering Singapore Singapore Date Posted Jun. 1, 2026 Deadline Open untill filled Po...</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/liz1ks87/Research-Fellow-Transportation-Engineering</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Civil, Construction and Environmental Engineering - Assistant Professor University of Alabama Civil, Construction and Environmental Engineering Tuscaloosa, Alabama United States Date Posted Jul. 29, 2</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>https://engineering.academickeys.com/job/02ixzgls/Civil-Construction-and-Environmental-Engineering--Assistant-Professor</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
@@ -853,73 +878,82 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>dfaed26f70dd7232</t>
+      <c r="O5" s="2" t="n">
+        <v>33.2120822</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>-87.53967350000001</v>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>f80ad2336a210f82</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Project Officer (TransportationEngineering)</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>AcademicKeys Listed Institution</t>
+          <t>University of Alabama</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering</t>
+          <t>Department of Civil, Construction and Environmental Engineering</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Civil Engineering, Construction Engineering, Environmental Engineering</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Tenured</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Review begins immediately / Open</t>
+          <t>Tuscaloosa, AL</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Project Officer ( Transportation Engineering) Nanyang Technological University School of Civil and Environmental Engineering Singapore Singapore Date Posted May 8, 2026 Deadline Open untill filled Pos...</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/in7p6mzx/Project-Officer-Transportation-Engineering</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>The University of Alabama seeks an Associate Professor in Civil, Construction, and Environmental Engineering holding a PhD in a related field. | Research Topics: Civil Engineering, Construction Engineering, Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>https://engineering.academickeys.com/job/w1r7nesq/Civil-Construction-and-Environmental-Engineering--Associate-Professor</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
@@ -927,46 +961,55 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>63eb9266e453efe9</t>
+      <c r="O6" s="2" t="n">
+        <v>33.2120822</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>-87.53967350000001</v>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>1b5f034d56841a04</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor of Civil Engineering</t>
+          <t>Assistant Professor of Urban Planning/Geography</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Cedarville University</t>
+          <t>Loyola Marymount University</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Civil &amp; Environmental / Transportation Engineering</t>
+          <t>Department of Urban and Environmental Studies</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Urban Planning, Geography, Environmental Studies</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Cedarville, OH</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -974,24 +1017,24 @@
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Assistant/Associate Professor of Civil Engineering Cedarville University Cedarville, OH Civil and Environmental Engineering Posted 10 days ago Priority</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179544290&amp;Title=Assistant%2FAssociate%20Professor%20of%20Civil%20Engineering</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>HigherEdJobs</t>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>$92,000</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Loyola Marymount University seeks a tenure-track Assistant Professor of Urban Planning/Geography with a relevant Ph.D. to conduct research and teach in the Department of Urban and Environmental Studies. | Research Topics: Urban Planning, Geography, Environmental Studies</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38031694/assistant-professor-of-urban-planning-geography/</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1001,50 +1044,55 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
-        <v>39.7540491</v>
-      </c>
       <c r="O7" s="2" t="n">
-        <v>-83.8170518</v>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>751c7406865a2787</t>
+        <v>33.9687824</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>-118.4182021</v>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>c13b0c3f0cf09a9e</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Assistant Professor of Urban Economics</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>University of Texas at Arlington</t>
+          <t>Harvard University</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Civil &amp; Environmental / Transportation Engineering</t>
+          <t>Harvard Kennedy School of Government</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Urban Economics, Regional Economics, Urban Policy</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Arlington, TX</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Cambridge, MA</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1052,24 +1100,24 @@
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Assistant Professor University of Texas at Arlington Arlington, TX Public Administration and Policy Posted Today</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179553472&amp;Title=Assistant%20Professor</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>HigherEdJobs</t>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>$165,000 - $185,000</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>The Harvard Kennedy School invites applications for a tenure-track Assistant Professor with a PhD in economics or a related field to study urgent issues affecting U.S. cities and regions. | Research Topics: Urban Economics, Regional Economics, Urban Policy</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38032116/assistant-professor-urban-economics-/</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1079,75 +1127,80 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
-        <v>32.7315155</v>
-      </c>
       <c r="O8" s="2" t="n">
-        <v>-97.1171533</v>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>85da23cbf7841060</t>
+        <v>42.3657432</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>-71.12221390000001</v>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>93251b0fa8170f49</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor, English (Film Studies and Contemporary U.S. Literature)</t>
+          <t>Assistant/Associate Professor of Civil Engineering (Transportation)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>University of Nevada Reno</t>
+          <t>Trine University</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Civil &amp; Environmental / Transportation Engineering</t>
+          <t>Reiners Department of Civil and Environmental Engineering</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>Transportation Engineering, Civil Engineering, Infrastructure Systems</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>Unspecified</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Reno, NV</t>
-        </is>
-      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Angola, IN</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>Open until filled</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Assistant Professor, English (Film Studies and Contemporary U.S. Literature) University of Nevada Reno Reno, NV $68,000 - $73,000 per year English and Literature Posted Today</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179553229&amp;Title=Assistant%20Professor%2C%20English%20%28Film%20Studies%20and%20Contemporary%20U%2ES%2E%20Literature%29</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>HigherEdJobs</t>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Based on qualifications</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Trine University is hiring a full-time Assistant or Associate Professor in Civil Engineering with a focus on transportation engineering, requiring a doctorate in civil engineering or a related field. | Research Topics: Transportation Engineering, Civil Engineering, Infrastructure Systems</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38028401/assistant-associate-professor-civil-engineering-transportation-/</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1157,50 +1210,55 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
-        <v>39.5442688</v>
-      </c>
       <c r="O9" s="2" t="n">
-        <v>-119.8163105</v>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>187a8dd6f5651753</t>
+        <v>41.6311141</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>-85.0105982</v>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>9f9cc58aa59ccd96</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Pharmaceutical Sciences - Drug Delivery</t>
+          <t>Adjunct Faculty - Transportation Engineering</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>University of Wisconsin - Madison</t>
+          <t>Morgan State University</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Civil &amp; Environmental / Transportation Engineering</t>
+          <t>School of Engineering</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Transportation Engineering, Traffic Flow, Transportation Systems</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Madison, WI</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Baltimore, MD</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1208,24 +1266,24 @@
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Assistant Professor of Pharmaceutical Sciences - Drug Delivery University of Wisconsin - Madison Madison, WI Pharmacy and Pharmacology Posted Today Military</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179553111&amp;Title=Assistant%20Professor%20of%20Pharmaceutical%20Sciences%20%2D%20Drug%20Delivery</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>HigherEdJobs</t>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Competitive Salary</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Morgan State University is seeking an Adjunct Faculty member to teach courses in Transportation Engineering, requiring at least a Master's or Ph.D. in a related discipline. | Research Topics: Transportation Engineering, Traffic Flow, Transportation Systems</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/37974518/adjunct-faculty-transportation-engineering/</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1235,50 +1293,55 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
-        <v>43.0802745</v>
-      </c>
       <c r="O10" s="2" t="n">
-        <v>-89.43095870000001</v>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>88a52598cec129d3</t>
+        <v>39.3446663</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>-76.5836094</v>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>3df6fb24b156d70b</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor of Metallurgical, Materials and Biomedical Engineering</t>
+          <t>Advanced Transportation Technology Instructor, Part-time Adjunct</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>University of Texas at El Paso</t>
+          <t>Kern Community College District</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Civil &amp; Environmental / Transportation Engineering</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Advanced Transportation Technology, Automotive Technology, Vehicle Systems</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>El Paso, TX</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>California</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1286,24 +1349,24 @@
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Assistant/Associate Professor of Metallurgical, Materials and Biomedical Engineering University of Texas at El Paso El Paso, TX Biological and Biomedical Engineering Posted Today</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179552602&amp;Title=Assistant%2FAssociate%20Professor%20of%20Metallurgical%2C%20Materials%20and%20Biomedical%20Engineering</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>HigherEdJobs</t>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>$65.00 Hourly</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Kern Community College District is seeking a Part-time Adjunct Instructor to teach advanced transportation technology courses. | Research Topics: Advanced Transportation Technology, Automotive Technology, Vehicle Systems</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38026829/advanced-transportation-technology-instructor-part-time-adjunct/</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1313,75 +1376,80 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
-        <v>31.7601001</v>
-      </c>
       <c r="O11" s="2" t="n">
-        <v>-106.4870476</v>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>a28cca356b9385b7</t>
+        <v>37.8719</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>-122.2585</v>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>36f117729bac62c9</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Urban Planning/Geography</t>
+          <t>Assistant/Associate/Full Professor, Transportation Engineering and Systems</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Chronicle Listed University</t>
+          <t>University of Cincinnati</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Transportation / Civil Engineering</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Transportation Engineering, Transportation Systems, Systems Engineering</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>See full listing</t>
+          <t>Cincinnati, OH</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Assistant Professor of Urban Planning/Geography Los Angeles, California (US) 92000 Loyola Marymount University Who We Are   The Department of Urban and Environmental Studies at Loyola Marymount Univer...</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38031694/assistant-professor-of-urban-planning-geography/</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Chronicle</t>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>The University of Cincinnati seeks an open-rank faculty member in Transportation Engineering and Systems, requiring a Ph.D. in civil engineering or a related field. | Research Topics: Transportation Engineering, Transportation Systems, Systems Engineering</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-transportation-engineering-and-systems-at-university-of-cincinnati-4416744025</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1391,71 +1459,80 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>c13b0c3f0cf09a9e</t>
+      <c r="O12" s="2" t="n">
+        <v>39.1318888</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>-84.51578309999999</v>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>6aa8ab000bc6f6c0</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor (Urban Economics)</t>
+          <t>Assistant/Associate Professor of Civil, Architectural and Environmental Engineering</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Chronicle Listed University</t>
+          <t>Missouri University of Science and Technology</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Transportation / Civil Engineering</t>
+          <t>Department of Civil, Architectural and Environmental Engineering</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Civil Engineering, Architectural Engineering, Environmental Engineering</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>See full listing</t>
+          <t>Rolla, MO</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Assistant Professor (Urban Economics) Cambridge, Massachusetts 165k - 185k Harvard Kennedy School of Government The Harvard Kennedy School invites applications for a junior economist who studies urgen...</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38032116/assistant-professor-urban-economics-/</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Chronicle</t>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Missouri University of Science and Technology invites applications for an Assistant/Associate Professor in Civil, Architectural and Environmental Engineering requiring a Ph.D. in a related engineering discipline. | Research Topics: Civil Engineering, Architectural Engineering, Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-associate-professor-civil-architectural-and-environmental-engineering-%2300096512-at-missouri-university-of-science-and-technology-4442271248</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1465,71 +1542,76 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>93251b0fa8170f49</t>
+      <c r="O13" s="2" t="n">
+        <v>37.9532435</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>-91.7742667</v>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>4fad8c46021c1243</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor - Civil Engineering (Transportation)</t>
+          <t>Assistant Professor – Urban Policy and Planning Dept., School of Arts and Sciences (Hunter College)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Chronicle Listed University</t>
+          <t>Hunter College</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Transportation / Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+          <t>Transportation Engineering</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Unspecified</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>See full listing</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
+          <t>Posted 2 months ago</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Assistant/Associate Professor - Civil Engineering (Transportation) Angola, Indiana Rank and salary will be based on qualifications. Trine University The Reiners Department of Civil and Environmental E...</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38028401/assistant-associate-professor-civil-engineering-transportation-/</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Chronicle</t>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assistant Professor – Urban Policy and Planning Dept., School of Arts and Sciences (Hunter College) Assistant Professor – Urban Policy and Planning Dept., School of Arts and Sciences (Hunter College) </t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-urban-policy-and-planning-dept-school-of-arts-and-sciences-hunter-college-at-hunter-college-4438624127</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1539,75 +1621,76 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>9f9cc58aa59ccd96</t>
+      <c r="O14" s="2" t="n">
+        <v>40.7683107</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>-73.964406</v>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>e4e18ed629103a27</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Transportation Driver</t>
+          <t>Research Assistant Professor - CYBER-CARE Consortium</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Chronicle Listed University</t>
+          <t>University of Houston</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Transportation / Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+          <t>Transportation Engineering</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Unspecified</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>See full listing</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
+          <t>Posted 4 months ago</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Transportation Driver Massachusetts, United States Salary Not specified College of the Holy Cross Transportation Driver
-College of the Holy Cross
-Part Time
-JREQ-000628
-At Holy Cross, we are focused ...</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38025514/transportation-driver/</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Chronicle</t>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Research Assistant Professor - CYBER-CARE Consortium Research Assistant Professor - CYBER-CARE Consortium University of Houston Houston, TX Be an early applicant 4 months ago</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/research-assistant-professor-cyber-care-consortium-at-university-of-houston-4404319276</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1617,73 +1700,76 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
-      <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>3d9a59d2266115bd</t>
+      <c r="O15" s="2" t="n">
+        <v>29.7207902</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>-95.34406269999999</v>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>c6ee2c0289357949</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Transportation Driver (Temporary)</t>
+          <t>Tenure-Track Faculty Position with a focus on Air Transportation Systems, Daytona Beach Campus</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Chronicle Listed University</t>
+          <t>Embry-Riddle Aeronautical University</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Transportation / Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+          <t>Transportation Engineering</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Unspecified</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>See full listing</t>
+          <t>Daytona Beach, FL</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
+          <t>Posted 1 month ago</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Transportation Driver (Temporary) Lancaster, California, United States Competitive Salary Antelope Valley College DESCRIPTION
-Under the direction of the Supervisor of Campus Events and/or
-designee pr...</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/37882967/transportation-driver-temporary-/</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Chronicle</t>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track Faculty Position with a focus on Air Transportation Systems, Daytona Beach Campus Tenure-Track Faculty Position with a focus on Air Transportation Systems, Daytona Beach Campus Embry-Ridd</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/tenure-track-faculty-position-with-a-focus-on-air-transportation-systems-daytona-beach-campus-at-embry-riddle-aeronautical-university-4434897662</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1693,402 +1779,21 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
-      <c r="O16" s="2" t="inlineStr"/>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>04d2e04a6ec65549</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Assistant/Associate/Full Professor, Transportation Engineering and Systems</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>University of Cincinnati</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Cincinnati, OH</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Posted 3 months ago</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Assistant/Associate/Full Professor, Transportation Engineering and Systems Assistant/Associate/Full Professor, Transportation Engineering and Systems University of Cincinnati Cincinnati, OH 3 months a...</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-transportation-engineering-and-systems-at-university-of-cincinnati-4416744025</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="n">
-        <v>39.1318888</v>
-      </c>
-      <c r="O17" s="2" t="n">
-        <v>-84.51578309999999</v>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>6aa8ab000bc6f6c0</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>ASSISTANT/ASSOCIATE PROFESSOR - Civil, Architectural and Environmental Engineering #00096512</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Missouri University of Science and Technology</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Rolla, MO</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Posted 1 week ago</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>ASSISTANT/ASSOCIATE PROFESSOR - Civil, Architectural and Environmental Engineering #00096512 ASSISTANT/ASSOCIATE PROFESSOR - Civil, Architectural and Environmental Engineering #00096512 Missouri Unive...</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-associate-professor-civil-architectural-and-environmental-engineering-%2300096512-at-missouri-university-of-science-and-technology-4442271248</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="n">
-        <v>37.9532435</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>-91.7742667</v>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>4fad8c46021c1243</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Assistant Professor – Urban Policy and Planning Dept., School of Arts and Sciences (Hunter College)</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Hunter College</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>New York, NY</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Posted 2 months ago</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Assistant Professor – Urban Policy and Planning Dept., School of Arts and Sciences (Hunter College) Assistant Professor – Urban Policy and Planning Dept., School of Arts and Sciences (Hunter College) ...</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-urban-policy-and-planning-dept-school-of-arts-and-sciences-hunter-college-at-hunter-college-4438624127</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="n">
-        <v>40.7683107</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>-73.964406</v>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>e4e18ed629103a27</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Research Assistant Professor - CYBER-CARE Consortium</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>University of Houston</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Houston, TX</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Posted 4 months ago</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Research Assistant Professor - CYBER-CARE Consortium Research Assistant Professor - CYBER-CARE Consortium University of Houston Houston, TX Be an early applicant 4 months ago</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/research-assistant-professor-cyber-care-consortium-at-university-of-houston-4404319276</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="n">
-        <v>29.7207902</v>
-      </c>
-      <c r="O20" s="2" t="n">
-        <v>-95.34406269999999</v>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>c6ee2c0289357949</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Tenure-Track Faculty Position with a focus on Air Transportation Systems, Daytona Beach Campus</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Embry-Riddle Aeronautical University</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Daytona Beach, FL</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Posted 1 month ago</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Tenure-Track Faculty Position with a focus on Air Transportation Systems, Daytona Beach Campus Tenure-Track Faculty Position with a focus on Air Transportation Systems, Daytona Beach Campus Embry-Ridd...</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/tenure-track-faculty-position-with-a-focus-on-air-transportation-systems-daytona-beach-campus-at-embry-riddle-aeronautical-university-4434897662</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="n">
+      <c r="O16" s="2" t="n">
         <v>33.8082375</v>
       </c>
-      <c r="O21" s="2" t="n">
+      <c r="P16" s="2" t="n">
         <v>-118.1344224</v>
       </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="Q16" s="2" t="inlineStr">
         <is>
           <t>b3c177958e0ab7a7</t>
         </is>
@@ -2096,26 +1801,21 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deduplicate by (institution, department) keeping latest update and expand geographic scope to US, Europe, HK, SG, JP, KR, TW (excluding Mainland China)
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -37,12 +37,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00276A3C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
@@ -50,6 +44,12 @@
     <font>
       <name val="Calibri"/>
       <color rgb="001F497D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00276A3C"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -68,14 +68,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00EDF2F8"/>
+        <bgColor rgb="00EDF2F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDF2F8"/>
-        <bgColor rgb="00EDF2F8"/>
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,17 +113,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S39"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -617,45 +617,45 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Transportation Engineering</t>
+          <t>Tenure-Track Faculty Position in Air Transportation Systems</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>University of Alabama</t>
+          <t>Chronicle Listed University</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Civil, Construction and Environmental Engineering</t>
+          <t>Air Transportation Systems (Daytona Beach Campus)</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Core match: position is explicitly for an Assistant Professor of Transportation Engineering.</t>
+          <t>Low fit: position focuses specifically on air transportation and aviation systems rather than ground transportation, transit, or mobility systems.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Traffic Operations, Intelligent Transportation Systems, Travel Behavior</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+          <t>Air Transportation Systems, Aviation, Transportation Management</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Tuscaloosa, AL</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
+          <t>Daytona Beach, FL</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -665,22 +665,22 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>The University of Alabama seeks a tenure-track Assistant Professor of Transportation Engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Transportation Engineering, Traffic Operations, Intelligent Transportation Systems, Travel Behavior</t>
-        </is>
-      </c>
-      <c r="L2" s="6" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/s9z6epb3/Civil-Construction-and-Environmental-Engineering--Transportation-Engineering--Assistant-Professor</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>AcademicKeys</t>
+          <t>This is a tenure-track faculty position focusing on air transportation systems at the Daytona Beach campus requiring an appropriate terminal degree. | Research Topics: Air Transportation Systems, Aviation, Transportation Management</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38012134/tenure-track-faculty-position-with-a-focus-on-air-transportation-systems-daytona-beach-campus/</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -688,63 +688,63 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>33.2120822</v>
+        <v>29.2108147</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>-87.53967350000001</v>
+        <v>-81.0228331</v>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>daabd65ea8fe188a</t>
+          <t>52969a207999417a</t>
         </is>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Transportation Engineering</t>
+          <t>Assistant Professor of Civil, Construction and Environmental Engineering</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>South Dakota State University</t>
+          <t>University of Alabama</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>10</v>
+          <t>Civil, Construction and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Core match: direct faculty position in Transportation Engineering aligning perfectly with the candidate's core field.</t>
+          <t>Broad Civil, Construction and Environmental Engineering faculty search where transportation is a potential sub-discipline within the department.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Traffic Systems, Infrastructure Planning, Smart Mobility</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
+          <t>Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Engineering</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Brookings, SD</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
+          <t>Tuscaloosa, AL</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -756,22 +756,22 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Assistant Professor position in Transportation Engineering requiring a Ph.D. in civil engineering or a closely related field to teach, advise, and conduct sponsored research. | Research Topics: Transportation Engineering, Traffic Systems, Infrastructure Planning, Smart Mobility</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/m4lk5asr/Assistant-Professor-of-Transportation-Engineering</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
+          <t>Assistant Professor position in the Department of Civil, Construction and Environmental Engineering at the University of Alabama. | Research Topics: Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Engineering</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>https://engineering.academickeys.com/job/02ixzgls/Civil-Construction-and-Environmental-Engineering--Assistant-Professor</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -779,63 +779,63 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>44.344449</v>
+        <v>33.2120822</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>-96.79823709999999</v>
+        <v>-87.53967350000001</v>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>9b7d5de4753a514b</t>
+          <t>f80ad2336a210f82</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor of Civil Engineering (Transportation)</t>
+          <t>Assistant Professor of Transportation Engineering</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Trine University</t>
+          <t>South Dakota State University</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>8</v>
+          <t>Department of Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>10</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Strong match for a tenure-track faculty position specifically in Civil Engineering with a focus on Transportation.</t>
+          <t>Core match: direct faculty position in Transportation Engineering aligning perfectly with the candidate's core field.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Civil Engineering Education, Mobility Systems</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
+          <t>Transportation Engineering, Traffic Systems, Infrastructure Planning, Smart Mobility</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Angola, IN</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
+          <t>Brookings, SD</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -847,15 +847,15 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>The role seeks a faculty member to teach and mentor undergraduate and graduate students in transportation engineering within a civil engineering department. | Research Topics: Transportation Engineering, Civil Engineering Education, Mobility Systems</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/e8akh47s/AssistantAssociate-Professor--Civil-Engineering-Transportation</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
+          <t>Assistant Professor position in Transportation Engineering requiring a Ph.D. in civil engineering or a closely related field to teach, advise, and conduct sponsored research. | Research Topics: Transportation Engineering, Traffic Systems, Infrastructure Planning, Smart Mobility</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>https://engineering.academickeys.com/job/m4lk5asr/Assistant-Professor-of-Transportation-Engineering</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
@@ -867,86 +867,86 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="P4" s="5" t="inlineStr">
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>41.6311141</v>
+        <v>44.344449</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>-85.0105982</v>
+        <v>-96.79823709999999</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>87a4115bef0ef2e7</t>
+          <t>9b7d5de4753a514b</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Urban Planning/Geography</t>
+          <t>Assistant/Associate Professor of Civil Engineering (Transportation)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Loyola Marymount University</t>
+          <t>Trine University</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Department of Urban Planning</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match in urban planning and geography with potential focus on urban mobility and transit systems.</t>
+          <t>Strong match for a faculty position specifically dedicated to transportation engineering within a civil engineering program.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Urban Planning, Geography, Mobility Systems, Urban Analytics</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+          <t>Transportation Engineering, Civil Engineering Education, Intelligent Transportation Systems</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
+          <t>Angola, IN</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>$92,000</t>
+          <t>Based on qualifications</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Assistant Professor position in urban planning and geography requiring a terminal degree in a relevant field to teach and conduct research. | Research Topics: Urban Planning, Geography, Mobility Systems, Urban Analytics</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38031694/assistant-professor-of-urban-planning-geography/</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
+          <t>This is a faculty position seeking a transportation engineering specialist to teach undergraduate and graduate civil engineering courses and mentor students. | Research Topics: Transportation Engineering, Civil Engineering Education, Intelligent Transportation Systems</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38028401/assistant-associate-professor-civil-engineering-transportation-/</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Chronicle</t>
         </is>
@@ -961,83 +961,83 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>33.9687824</v>
+        <v>41.6311141</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>-118.4182021</v>
+        <v>-85.0105982</v>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>c13b0c3f0cf09a9e</t>
+          <t>9f9cc58aa59ccd96</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Urban Economics</t>
+          <t>Assistant Professor of Urban Planning/Geography</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Harvard University</t>
+          <t>Loyola Marymount University</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Department of Economics / Graduate School of Design</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>5</v>
+          <t>Department of Urban Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: urban economics position focusing on economic analysis rather than core transportation engineering and travel behavior.</t>
+          <t>Strong interdisciplinary match in urban planning and geography with potential focus on urban mobility and transit systems.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Urban Economics, Spatial Economics, Urban Analytics, Real Estate and Housing</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+          <t>Urban Planning, Geography, Mobility Systems, Urban Analytics</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Cambridge, MA</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>$165,000 - $185,000</t>
+          <t>$92,000</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track faculty role in urban economics requiring a Ph.D. in economics, public policy, or a closely related field with a focus on urban systems. | Research Topics: Urban Economics, Spatial Economics, Urban Analytics, Real Estate and Housing</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38032116/assistant-professor-urban-economics-/</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
+          <t>Assistant Professor position in urban planning and geography requiring a terminal degree in a relevant field to teach and conduct research. | Research Topics: Urban Planning, Geography, Mobility Systems, Urban Analytics</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38031694/assistant-professor-of-urban-planning-geography/</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>Chronicle</t>
         </is>
@@ -1052,83 +1052,83 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>42.3657432</v>
+        <v>33.9687824</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>-71.12221390000001</v>
+        <v>-118.4182021</v>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>93251b0fa8170f49</t>
+          <t>c13b0c3f0cf09a9e</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor of Civil Engineering (Transportation)</t>
+          <t>Assistant Professor of Urban Economics</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Trine University</t>
+          <t>Harvard University</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>8</v>
+          <t>Department of Economics / Graduate School of Design</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Strong match for a faculty position specifically dedicated to transportation engineering within a civil engineering program.</t>
+          <t>Moderate fit: urban economics position focusing on economic analysis rather than core transportation engineering and travel behavior.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Civil Engineering Education, Intelligent Transportation Systems</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
+          <t>Urban Economics, Spatial Economics, Urban Analytics, Real Estate and Housing</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Angola, IN</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
+          <t>Cambridge, MA</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Based on qualifications</t>
+          <t>$165,000 - $185,000</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>This is a faculty position seeking a transportation engineering specialist to teach undergraduate and graduate civil engineering courses and mentor students. | Research Topics: Transportation Engineering, Civil Engineering Education, Intelligent Transportation Systems</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38028401/assistant-associate-professor-civil-engineering-transportation-/</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
+          <t>This is a tenure-track faculty role in urban economics requiring a Ph.D. in economics, public policy, or a closely related field with a focus on urban systems. | Research Topics: Urban Economics, Spatial Economics, Urban Analytics, Real Estate and Housing</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38032116/assistant-professor-urban-economics-/</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Chronicle</t>
         </is>
@@ -1143,20 +1143,20 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P7" s="5" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>41.6311141</v>
+        <v>42.3657432</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>-85.0105982</v>
+        <v>-71.12221390000001</v>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>9f9cc58aa59ccd96</t>
+          <t>93251b0fa8170f49</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
           <t>Civil and Environmental Engineering</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="7" t="n">
         <v>9</v>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1189,7 +1189,7 @@
           <t>Transportation Engineering, Transit Planning, Traffic Systems</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Non-Tenure Track</t>
         </is>
@@ -1199,7 +1199,7 @@
           <t>Baltimore, MD</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -1214,12 +1214,12 @@
           <t>The role seeks an adjunct faculty member to teach transportation engineering courses within the civil and environmental engineering department, requiring a relevant graduate degree. | Research Topics: Transportation Engineering, Transit Planning, Traffic Systems</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>https://jobs.chronicle.com/job/37974518/adjunct-faculty-transportation-engineering/</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>Chronicle</t>
         </is>
@@ -1234,7 +1234,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1267,7 +1267,7 @@
           <t>Advanced Transportation Technology</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1280,7 +1280,7 @@
           <t>Advanced Transportation Technology, Vehicle Technologies, Transportation Education</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Non-Tenure Track</t>
         </is>
@@ -1290,7 +1290,7 @@
           <t>California</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -1305,12 +1305,12 @@
           <t>Part-time adjunct instructor role teaching advanced transportation technology courses at a community college district. | Research Topics: Advanced Transportation Technology, Vehicle Technologies, Transportation Education</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>https://jobs.chronicle.com/job/38026829/advanced-transportation-technology-instructor-part-time-adjunct/</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>Chronicle</t>
         </is>
@@ -1325,7 +1325,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P9" s="5" t="inlineStr">
+      <c r="P9" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1358,7 +1358,7 @@
           <t>Department of Civil and Architectural Engineering and Construction Management</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="7" t="n">
         <v>10</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1371,7 +1371,7 @@
           <t>Transportation Engineering, Transportation Systems, Transit Planning, Mobility Systems</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -1381,7 +1381,7 @@
           <t>Cincinnati, OH</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -1396,12 +1396,12 @@
           <t>The Department of Civil and Architectural Engineering and Construction Management at the University of Cincinnati is seeking an open-rank faculty member specializing in transportation engineering and systems. | Research Topics: Transportation Engineering, Transportation Systems, Transit Planning, Mobility Systems</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-transportation-engineering-and-systems-at-university-of-cincinnati-4416744025</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -1416,7 +1416,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P10" s="5" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1449,7 +1449,7 @@
           <t>Civil, Architectural and Environmental Engineering</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1462,7 +1462,7 @@
           <t>Civil Engineering, Architectural Engineering, Environmental Engineering</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -1472,7 +1472,7 @@
           <t>Rolla, MO</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -1487,12 +1487,12 @@
           <t>The position seeks an Assistant or Associate Professor in the Department of Civil, Architectural and Environmental Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Civil Engineering, Architectural Engineering, Environmental Engineering</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/assistant-associate-professor-civil-architectural-and-environmental-engineering-%2300096512-at-missouri-university-of-science-and-technology-4442271248</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -1507,7 +1507,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P11" s="5" t="inlineStr">
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1540,7 +1540,7 @@
           <t>Department of Urban Policy and Planning, School of Arts and Sciences</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="7" t="n">
         <v>8</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1553,7 +1553,7 @@
           <t>Transportation Policy, Transit Accessibility, Transportation Equity, Community-Engaged Research</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -1563,7 +1563,7 @@
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Open until filled (Review begins Oct. 1, 2025)</t>
         </is>
@@ -1578,12 +1578,12 @@
           <t>Hunter College seeks a tenure-track Assistant Professor in transportation policy requiring a Ph.D. in policy, planning, or a related field to teach applied policy research and develop a robust research agenda. | Research Topics: Transportation Policy, Transit Accessibility, Transportation Equity, Community-Engaged Research</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-urban-policy-and-planning-dept-school-of-arts-and-sciences-hunter-college-at-hunter-college-4438624127</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -1598,7 +1598,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P12" s="5" t="inlineStr">
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1631,7 +1631,7 @@
           <t>Information Science Technology (CYBER-CARE Consortium)</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1644,7 +1644,7 @@
           <t>Connected and Automated Vehicle Cybersecurity, Transportation Data Security, Advanced Traffic Management Systems, Intelligent Transportation Systems</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Non-Tenure Track</t>
         </is>
@@ -1654,7 +1654,7 @@
           <t>Houston, TX</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -1669,12 +1669,12 @@
           <t>The University of Houston seeks a non-tenure track Research Assistant Professor for the CYBER-CARE consortium to conduct research on transportation cybersecurity and AI applications, requiring a doctoral degree in Transportation Engineering or a closely related field. | Research Topics: Connected and Automated Vehicle Cybersecurity, Transportation Data Security, Advanced Traffic Management Systems, Intelligent Transportation Systems</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="L13" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/research-assistant-professor-cyber-care-consortium-at-university-of-houston-4404319276</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -1689,7 +1689,7 @@
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="P13" s="5" t="inlineStr">
+      <c r="P13" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1722,7 +1722,7 @@
           <t>School of Graduate Studies in the College of Aviation</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="3" t="n">
         <v>4</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1735,7 +1735,7 @@
           <t>Air Transportation Systems, Advanced Air Mobility, UAS Traffic Management, Machine Learning/AI in Aviation</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -1745,7 +1745,7 @@
           <t>Daytona Beach, FL</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>Review begins immediately; Priority given to applications received by 2026-08-31</t>
         </is>
@@ -1760,12 +1760,12 @@
           <t>This tenure-track faculty position requires a doctorate in air transportation systems, advanced air mobility, or a related area to teach graduate courses and conduct AI/machine learning research in aviation. | Research Topics: Air Transportation Systems, Advanced Air Mobility, UAS Traffic Management, Machine Learning/AI in Aviation</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="L14" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/tenure-track-faculty-position-with-a-focus-on-air-transportation-systems-daytona-beach-campus-at-embry-riddle-aeronautical-university-4434897662</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -1780,7 +1780,7 @@
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="P14" s="5" t="inlineStr">
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1800,7 +1800,7 @@
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor / Associate Professor in Maritime Studies</t>
+          <t>Assistant Professor / Associate Professor (Tenure-Track) in Civil and Environmental Engineering</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1813,30 +1813,30 @@
           <t>School of Civil and Environmental Engineering</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: maritime studies includes ports and logistics, but the focus is broader than the candidate's core transportation engineering specialization.</t>
+          <t>Moderate fit: broad Civil and Environmental Engineering search where Transportation Engineering is a potential sub-discipline, though specific subfield requirements are not detailed in the snippet.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Maritime Studies, Port Logistics, Transportation Systems, Supply Chain</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
+          <t>Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
+          <t>Singapore, Singapore</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -1848,22 +1848,22 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>This is a faculty position focusing on maritime studies and port-related systems, requiring a relevant Ph.D. degree. | Research Topics: Maritime Studies, Port Logistics, Transportation Systems, Supply Chain</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/m80x7utf/Assistant-Professor--Associate-Professor-TenureTrack-Associate-Professor-PracticeTrack-in-Maritime-Studies</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
+          <t>Tenure-track Assistant or Associate Professor position in Civil and Environmental Engineering requiring an earned doctorate in civil engineering or a closely related discipline. | Research Topics: Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>https://engineering.academickeys.com/job/dhzin0q4/Assistant-Professor--Associate-Professor-TenureTrack-in-Civil-and-Environmental-Engineering</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -1871,20 +1871,20 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P15" s="5" t="inlineStr">
+      <c r="P15" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>1.357107</v>
+        <v>1.2899175</v>
       </c>
       <c r="R15" s="2" t="n">
-        <v>103.8194992</v>
+        <v>103.8519072</v>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>6736da1a934c5c83</t>
+          <t>3fa57c30724444e8</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
           <t>Department of Mechanical Engineering</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1917,7 +1917,7 @@
           <t>Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -1927,7 +1927,7 @@
           <t>Auburn, AL</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
@@ -1942,12 +1942,12 @@
           <t>An open-rank faculty position in mechanical engineering requiring a Ph.D. in mechanical engineering or a closely related field. | Research Topics: Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t>https://engineering.academickeys.com/job/f320isty/AssistantAssociateFull-Professor</t>
         </is>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
@@ -1962,7 +1962,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P16" s="5" t="inlineStr">
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1995,7 +1995,7 @@
           <t>Industrial and Systems Engineering</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="6" t="n">
         <v>7</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -2008,7 +2008,7 @@
           <t>Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -2018,7 +2018,7 @@
           <t>Seattle, WA</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Unspecified</t>
         </is>
@@ -2033,12 +2033,12 @@
           <t>Assistant or Associate Professor position in Industrial and Systems Engineering requiring a Ph.D. in a relevant engineering or analytical discipline. | Research Topics: Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr">
         <is>
           <t>https://engineering.academickeys.com/job/g4m97a60/AssistantAssociate-Professor-Industrial-and-Systems-Engineering-Systems-Engineering-Focus</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
@@ -2053,7 +2053,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P17" s="5" t="inlineStr">
+      <c r="P17" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2086,7 +2086,7 @@
           <t>Department of Civil and Environmental Engineering</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -2099,7 +2099,7 @@
           <t>Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Tenured</t>
         </is>
@@ -2109,7 +2109,7 @@
           <t>Pittsburgh, PA</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -2124,12 +2124,12 @@
           <t>Strictly 1 concise sentence summarizing the primary focus of the role and minimum degree qualification. | Research Topics: Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L18" s="5" t="inlineStr">
         <is>
           <t>http://engineering.academickeys.com/job/vhlo0w6p/Professor--Department-Chair--Electrical-and-Computer-Engineering</t>
         </is>
       </c>
-      <c r="M18" s="5" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
@@ -2144,7 +2144,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P18" s="5" t="inlineStr">
+      <c r="P18" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2177,7 +2177,7 @@
           <t>Not specified</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -2190,7 +2190,7 @@
           <t>Higher Education, Instruction, Academic Teaching</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Non-Tenure Track</t>
         </is>
@@ -2200,7 +2200,7 @@
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
@@ -2215,12 +2215,12 @@
           <t>This is a faculty teaching role at Columbia University, though the specific academic department and subject focus are missing from the current snippet. | Research Topics: Higher Education, Instruction, Academic Teaching</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L19" s="5" t="inlineStr">
         <is>
           <t>http://engineering.academickeys.com/job/arsy3jqh/Open-Rank-Lecturer-in-Discipline-or-Senior-Lecturer-in-Discipline</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>AcademicKeys</t>
         </is>
@@ -2235,7 +2235,7 @@
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="P19" s="5" t="inlineStr">
+      <c r="P19" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2268,7 +2268,7 @@
           <t>Department of Civil Engineering</t>
         </is>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2281,7 +2281,7 @@
           <t>Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -2291,7 +2291,7 @@
           <t>Cedarville, OH</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
@@ -2306,12 +2306,12 @@
           <t>A faculty position in civil engineering requiring a Ph.D. to teach undergraduate courses and engage in scholarly activity. | Research Topics: Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="L20" s="5" t="inlineStr">
         <is>
           <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179544290&amp;Title=Assistant%2FAssociate%20Professor%20of%20Civil%20Engineering</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="M20" s="3" t="inlineStr">
         <is>
           <t>HigherEdJobs</t>
         </is>
@@ -2326,7 +2326,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P20" s="5" t="inlineStr">
+      <c r="P20" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2359,7 +2359,7 @@
           <t>Information and Decision Sciences (IDS)</t>
         </is>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -2372,7 +2372,7 @@
           <t>Supply Chain Management, Operations Management, Decision Sciences</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -2382,7 +2382,7 @@
           <t>Chicago, IL</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -2397,12 +2397,12 @@
           <t>This is a tenure-track Assistant Professor role in Supply Chain and Operations Management requiring a Ph.D. in a relevant business or analytical discipline. | Research Topics: Supply Chain Management, Operations Management, Decision Sciences</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="L21" s="5" t="inlineStr">
         <is>
           <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179552436&amp;Title=Assistant%20Professor%20%2D%20IDS%20%28Supply%20Chain%20%26%20Operations%20Management%29</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>HigherEdJobs</t>
         </is>
@@ -2417,7 +2417,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P21" s="5" t="inlineStr">
+      <c r="P21" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2450,7 +2450,7 @@
           <t>Department of Industrial and Systems Engineering</t>
         </is>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="6" t="n">
         <v>6</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -2463,7 +2463,7 @@
           <t>Industrial Engineering, Systems Engineering, Operations Research</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -2473,7 +2473,7 @@
           <t>Auburn, AL</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -2488,12 +2488,12 @@
           <t>Open-rank faculty position in Industrial and Systems Engineering requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Systems Engineering, Operations Research</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="L22" s="5" t="inlineStr">
         <is>
           <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179548357&amp;Title=Professor%2C%20Associate%20Professor%2C%20Assistant%20Professor%20%2D%20Industrial%20and%20Systems%20Engineering</t>
         </is>
       </c>
-      <c r="M22" s="5" t="inlineStr">
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>HigherEdJobs</t>
         </is>
@@ -2508,7 +2508,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P22" s="5" t="inlineStr">
+      <c r="P22" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2541,7 +2541,7 @@
           <t>Department of Industrial and Systems Engineering</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="6" t="n">
         <v>7</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -2554,7 +2554,7 @@
           <t>Industrial Engineering, Mobility Systems, Systems Engineering</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
@@ -2564,7 +2564,7 @@
           <t>Knoxville, TN</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -2579,12 +2579,12 @@
           <t>Tenure-track Assistant Professor position in Industrial and Systems Engineering focusing on mobility systems, requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Mobility Systems, Systems Engineering</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
         <is>
           <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545449&amp;Title=Tenure%2DTrack%20Assistant%20Professor%20of%20Industrial%20and%20Systems%20Engineering%2C%20Fall%202027%20%281%2F3%29</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="M23" s="3" t="inlineStr">
         <is>
           <t>HigherEdJobs</t>
         </is>
@@ -2599,7 +2599,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P23" s="5" t="inlineStr">
+      <c r="P23" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2632,7 +2632,7 @@
           <t>Civil Engineering</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -2645,7 +2645,7 @@
           <t>Civil Engineering Education, Transportation Engineering</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Non-Tenure Track</t>
         </is>
@@ -2655,7 +2655,7 @@
           <t>Fayetteville, AR</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -2670,12 +2670,12 @@
           <t>A teaching-focused assistant professor position in civil engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Civil Engineering Education, Transportation Engineering</t>
         </is>
       </c>
-      <c r="L24" s="6" t="inlineStr">
+      <c r="L24" s="5" t="inlineStr">
         <is>
           <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179541925&amp;Title=Teaching%20Assistant%20Professor</t>
         </is>
       </c>
-      <c r="M24" s="5" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>HigherEdJobs</t>
         </is>
@@ -2690,7 +2690,7 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P24" s="5" t="inlineStr">
+      <c r="P24" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2710,65 +2710,65 @@
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Tenure-Track Faculty Position in Air Transportation Systems</t>
+          <t>Assistant Professor of Teaching</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Chronicle Listed University</t>
+          <t>Florida Atlantic University</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Air Transportation Systems (Daytona Beach Campus)</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>3</v>
+          <t>Department of Civil, Environmental &amp; Geomatics Engineering</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Low fit: position focuses specifically on air transportation and aviation systems rather than ground transportation, transit, or mobility systems.</t>
+          <t>Moderate fit: it is a Civil Engineering teaching position in a department with transportation research centers, but requires teaching structural analysis and design-related classes alongside a P.E. license.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Air Transportation Systems, Aviation, Transportation Management</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Tenure-Track</t>
+          <t>Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Daytona Beach, FL</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>Not specified</t>
+          <t>Boca Raton, FL</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Commensurate with Experience</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track faculty position focusing on air transportation systems at the Daytona Beach campus requiring an appropriate terminal degree. | Research Topics: Air Transportation Systems, Aviation, Transportation Management</t>
-        </is>
-      </c>
-      <c r="L25" s="6" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38012134/tenure-track-faculty-position-with-a-focus-on-air-transportation-systems-daytona-beach-campus/</t>
-        </is>
-      </c>
-      <c r="M25" s="5" t="inlineStr">
-        <is>
-          <t>Chronicle</t>
+          <t>This is a non-tenure-track Assistant Teaching Professor position in civil engineering requiring a Ph.D. and P.E. license to teach undergraduate and graduate courses including structural analysis and design. | Research Topics: Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-teaching-at-florida-atlantic-university-4414964381</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -2778,86 +2778,86 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P25" s="5" t="inlineStr">
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>29.2108147</v>
+        <v>26.1194058</v>
       </c>
       <c r="R25" s="2" t="n">
-        <v>-81.0228331</v>
+        <v>-80.14167999999999</v>
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>52969a207999417a</t>
+          <t>7bdaa996cf64d1f6</t>
         </is>
       </c>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Teaching</t>
+          <t>Assistant or Associate Professor in Supply Chain Management</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Florida Atlantic University</t>
+          <t>University of Arkansas</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil, Environmental &amp; Geomatics Engineering</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="n">
-        <v>5</v>
+          <t>J.B. Hunt Transport Department of Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: it is a Civil Engineering teaching position in a department with transportation research centers, but requires teaching structural analysis and design-related classes alongside a P.E. license.</t>
+          <t>Low fit: this is a faculty position in Supply Chain Management within a Business School rather than Transportation Engineering.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>Non-Tenure Track</t>
+          <t>Supply Chain Management, Logistics, Operations Research</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Boca Raton, FL</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
+          <t>Fayetteville, AR</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Commensurate with Experience</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>This is a non-tenure-track Assistant Teaching Professor position in civil engineering requiring a Ph.D. and P.E. license to teach undergraduate and graduate courses including structural analysis and design. | Research Topics: Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
-        </is>
-      </c>
-      <c r="L26" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-teaching-at-florida-atlantic-university-4414964381</t>
-        </is>
-      </c>
-      <c r="M26" s="5" t="inlineStr">
+          <t>This is a tenure-track Assistant or Associate Professor position in Supply Chain Management requiring a strong research record in leading peer-reviewed journals. | Research Topics: Supply Chain Management, Logistics, Operations Research</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-or-associate-professor-open-rank-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460111187</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -2869,68 +2869,68 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="P26" s="5" t="inlineStr">
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>26.1194058</v>
+        <v>36.0625843</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>-80.14167999999999</v>
+        <v>-94.1574328</v>
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>7bdaa996cf64d1f6</t>
+          <t>c16a694d5f7f68d4</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Assistant or Associate Professor in Supply Chain Management</t>
+          <t>Assistant Professor of Aerospace Engineering</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>The University of Kansas</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>J.B. Hunt Transport Department of Supply Chain Management</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="n">
+          <t>Department of Aerospace Engineering</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Low fit: this is a faculty position in Supply Chain Management within a Business School rather than Transportation Engineering.</t>
+          <t>The position is specifically for Aerospace Engineering focusing on aircraft and space systems, where the candidate's core transportation engineering expertise is not the primary requirement.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Logistics, Operations Research</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
+          <t>Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
+          <t>Lawrence, KS</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2940,15 +2940,15 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track Assistant or Associate Professor position in Supply Chain Management requiring a strong research record in leading peer-reviewed journals. | Research Topics: Supply Chain Management, Logistics, Operations Research</t>
-        </is>
-      </c>
-      <c r="L27" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-or-associate-professor-open-rank-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460111187</t>
-        </is>
-      </c>
-      <c r="M27" s="5" t="inlineStr">
+          <t>This is a tenure-track faculty position in Aerospace Engineering requiring a doctorate in Aerospace Engineering or a closely related field, focusing on aviation and space-related research. | Research Topics: Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-aerospace-engineering-at-the-university-of-kansas-4460398978</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -2963,83 +2963,83 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P27" s="5" t="inlineStr">
+      <c r="P27" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>36.0625843</v>
+        <v>39.0559267</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>-94.1574328</v>
+        <v>-94.6090332</v>
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>c16a694d5f7f68d4</t>
+          <t>4a53cfad86712a72</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Aerospace Engineering</t>
+          <t>Assistant/Associate/Full Professor in Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>The University of Kansas</t>
+          <t>University of Florida</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Department of Aerospace Engineering</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="n">
-        <v>3</v>
+          <t>Department of Industrial and Systems Engineering</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>The position is specifically for Aerospace Engineering focusing on aircraft and space systems, where the candidate's core transportation engineering expertise is not the primary requirement.</t>
+          <t>Moderate fit: while housed in Industrial and Systems Engineering with a broad mention of transportation applications, the primary departmental focus and hiring emphasis is strictly on Industrialized Construction.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
+          <t>Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Lawrence, KS</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
+          <t>Gainesville, FL</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track faculty position in Aerospace Engineering requiring a doctorate in Aerospace Engineering or a closely related field, focusing on aviation and space-related research. | Research Topics: Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
-        </is>
-      </c>
-      <c r="L28" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-aerospace-engineering-at-the-university-of-kansas-4460398978</t>
-        </is>
-      </c>
-      <c r="M28" s="5" t="inlineStr">
+          <t>The Department of Industrial and Systems Engineering at the University of Florida seeks a tenured/tenure-track faculty member specializing in Industrialized Construction with a PhD in ISE, Manufacturing Engineering, Civil Engineering, Mechanical Engineering, or a closely related field. | Research Topics: Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-industrial-systems-engineering-at-university-of-florida-4323668785</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -3051,68 +3051,68 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P28" s="5" t="inlineStr">
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>39.0559267</v>
+        <v>29.6436</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>-94.6090332</v>
+        <v>-82.3549</v>
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>4a53cfad86712a72</t>
+          <t>56d501f448e77e05</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate/Full Professor in Industrial and Systems Engineering</t>
+          <t>Assistant Professor in Supply Chain Management</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>University of Florida</t>
+          <t>University of Arkansas</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial and Systems Engineering</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>4</v>
+          <t>J.B. Hunt Transport Department of Supply Chain Management, Sam M. Walton College of Business</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: while housed in Industrial and Systems Engineering with a broad mention of transportation applications, the primary departmental focus and hiring emphasis is strictly on Industrialized Construction.</t>
+          <t>Low fit: Business school faculty position focused entirely on defense-relevant supply chain management and contested logistics, which falls outside transportation engineering.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
+          <t>Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Gainesville, FL</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
+          <t>Fayetteville, AR</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -3122,15 +3122,15 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>The Department of Industrial and Systems Engineering at the University of Florida seeks a tenured/tenure-track faculty member specializing in Industrialized Construction with a PhD in ISE, Manufacturing Engineering, Civil Engineering, Mechanical Engineering, or a closely related field. | Research Topics: Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
-        </is>
-      </c>
-      <c r="L29" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-industrial-systems-engineering-at-university-of-florida-4323668785</t>
-        </is>
-      </c>
-      <c r="M29" s="5" t="inlineStr">
+          <t>The Sam M. Walton College of Business at the University of Arkansas seeks two tenure-track Assistant Professors in Supply Chain Management as part of a faculty cluster hire focused on contested logistics and defense-relevant supply chains. | Research Topics: Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-two-open-positions-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460109211</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -3142,23 +3142,23 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="P29" s="5" t="inlineStr">
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>29.6436</v>
+        <v>36.0625843</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>-82.3549</v>
+        <v>-94.1574328</v>
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>56d501f448e77e05</t>
+          <t>8b974c86c7dfa1c1</t>
         </is>
       </c>
     </row>
@@ -3170,40 +3170,40 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>Iowa State University</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>J.B. Hunt Transport Department of Supply Chain Management, Sam M. Walton College of Business</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="n">
-        <v>3</v>
+          <t>Department of Supply Chain Management, Ivy College of Business</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Low fit: Business school faculty position focused entirely on defense-relevant supply chain management and contested logistics, which falls outside transportation engineering.</t>
+          <t>Moderate fit: the role is in a business school supply chain department rather than engineering or planning, though it accepts transportation as a related specialization.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
+          <t>Supply Chain Management, Transportation, Logistics, Operations</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
+          <t>Ames, IA</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3213,15 +3213,15 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>The Sam M. Walton College of Business at the University of Arkansas seeks two tenure-track Assistant Professors in Supply Chain Management as part of a faculty cluster hire focused on contested logistics and defense-relevant supply chains. | Research Topics: Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
-        </is>
-      </c>
-      <c r="L30" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-two-open-positions-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460109211</t>
-        </is>
-      </c>
-      <c r="M30" s="5" t="inlineStr">
+          <t>The Ivy College of Business at Iowa State University seeks a tenure-track Assistant Professor in Supply Chain Management to conduct research and teach across undergraduate, master's, and Ph.D. levels, requiring a Ph.D. in business administration or a related field such as transportation or logistics. | Research Topics: Supply Chain Management, Transportation, Logistics, Operations</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-in-supply-chain-management-at-iowa-state-university-ivy-college-of-business-4440811209</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -3233,86 +3233,86 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P30" s="5" t="inlineStr">
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>36.0625843</v>
+        <v>42.0267567</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>-94.1574328</v>
+        <v>-93.6170448</v>
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>8b974c86c7dfa1c1</t>
+          <t>e994e392d38b77ce</t>
         </is>
       </c>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Supply Chain Management</t>
+          <t>Assistant Professor in Operations Management</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Iowa State University</t>
+          <t>University of Illinois Chicago</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Department of Supply Chain Management, Ivy College of Business</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>6</v>
+          <t>Department of Information and Decision Sciences, College of Business Administration</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: the role is in a business school supply chain department rather than engineering or planning, though it accepts transportation as a related specialization.</t>
+          <t>Strong interdisciplinary match in a Business School department that explicitly prioritizes transportation and AI in supply chain management as a preferred research domain.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Transportation, Logistics, Operations</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
+          <t>Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Ames, IA</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>2026-12-06</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$185,000 - $220,000 annually</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>The Ivy College of Business at Iowa State University seeks a tenure-track Assistant Professor in Supply Chain Management to conduct research and teach across undergraduate, master's, and Ph.D. levels, requiring a Ph.D. in business administration or a related field such as transportation or logistics. | Research Topics: Supply Chain Management, Transportation, Logistics, Operations</t>
-        </is>
-      </c>
-      <c r="L31" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-in-supply-chain-management-at-iowa-state-university-ivy-college-of-business-4440811209</t>
-        </is>
-      </c>
-      <c r="M31" s="5" t="inlineStr">
+          <t>The Department of Information and Decision Sciences seeks a tenure-track Assistant Professor in Operations Management with a preferred research focus on transportation and AI-driven supply chain management, requiring a Ph.D. in Management Science, Operations Management, Operations Research, or a closely related field. | Research Topics: Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-ids-supply-chain-operations-management-at-university-of-illinois-chicago-4463632919</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -3327,83 +3327,83 @@
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="P31" s="5" t="inlineStr">
+      <c r="P31" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>42.0267567</v>
+        <v>41.8748613</v>
       </c>
       <c r="R31" s="2" t="n">
-        <v>-93.6170448</v>
+        <v>-87.6519866</v>
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>e994e392d38b77ce</t>
+          <t>d58da246ce5b68ab</t>
         </is>
       </c>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Operations Management</t>
+          <t>Assistant Professor of Public Policy (Market-Based Solutions to Societal Challenges)</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>University of Illinois Chicago</t>
+          <t>University of Wisconsin-Madison</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Department of Information and Decision Sciences, College of Business Administration</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="n">
-        <v>7</v>
+          <t>La Follette School of Public Affairs, College of Letters &amp; Science</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match in a Business School department that explicitly prioritizes transportation and AI in supply chain management as a preferred research domain.</t>
+          <t>Low fit: Public policy and economics faculty position focused on market-based solutions, though transportation and infrastructure finance is listed as one of many broad application areas.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
+          <t>Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>2026-12-06</t>
+          <t>Madison, WI</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>$185,000 - $220,000 annually</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>The Department of Information and Decision Sciences seeks a tenure-track Assistant Professor in Operations Management with a preferred research focus on transportation and AI-driven supply chain management, requiring a Ph.D. in Management Science, Operations Management, Operations Research, or a closely related field. | Research Topics: Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
-        </is>
-      </c>
-      <c r="L32" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-ids-supply-chain-operations-management-at-university-of-illinois-chicago-4463632919</t>
-        </is>
-      </c>
-      <c r="M32" s="5" t="inlineStr">
+          <t>The La Follette School of Public Affairs at UW-Madison seeks a tenure-track assistant professor to conduct theoretically grounded research on market-based solutions and incentive-compatible policy design across various domains. | Research Topics: Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-public-policy-market-based-solutions-to-societal-challenges-at-uw-madison-college-of-letters-science-4435310692</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
@@ -3415,66 +3415,66 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="P32" s="5" t="inlineStr">
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>41.8748613</v>
+        <v>43.07469</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>-87.6519866</v>
+        <v>-89.3841663</v>
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>d58da246ce5b68ab</t>
+          <t>886b76b05d362fdc</t>
         </is>
       </c>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Public Policy (Market-Based Solutions to Societal Challenges)</t>
+          <t>Multiple Faculty Positions in Computer Science and Engineering</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Madison</t>
+          <t>Texas A&amp;M University</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>La Follette School of Public Affairs, College of Letters &amp; Science</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="n">
-        <v>3</v>
+          <t>Department of Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Low fit: Public policy and economics faculty position focused on market-based solutions, though transportation and infrastructure finance is listed as one of many broad application areas.</t>
+          <t>Moderate fit: open faculty search in Computer Science and Engineering without explicit specialization in transportation or mobility systems.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>Tenure-Track</t>
+          <t>Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Madison, WI</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
+          <t>College Station, TX</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
@@ -3486,22 +3486,22 @@
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>The La Follette School of Public Affairs at UW-Madison seeks a tenure-track assistant professor to conduct theoretically grounded research on market-based solutions and incentive-compatible policy design across various domains. | Research Topics: Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
-        </is>
-      </c>
-      <c r="L33" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-public-policy-market-based-solutions-to-societal-challenges-at-uw-madison-college-of-letters-science-4435310692</t>
-        </is>
-      </c>
-      <c r="M33" s="5" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
+          <t>Texas A&amp;M University invites applications for multiple faculty positions in Computer Science and Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>http://engineering.academickeys.com/job/rh7lvag4/CSE--TAMU-Multiple-Faculty-Positions</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -3509,85 +3509,85 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P33" s="5" t="inlineStr">
+      <c r="P33" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>43.07469</v>
+        <v>30.6187</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>-89.3841663</v>
+        <v>-96.3365</v>
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>886b76b05d362fdc</t>
+          <t>7d5d844d65485b4b</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Civil, Construction and Environmental Engineering</t>
+          <t>Assistant Professor of Civil Engineering</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>University of Alabama</t>
+          <t>McNeese State University</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Civil, Construction and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="n">
-        <v>6</v>
+          <t>Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Broad Civil, Construction and Environmental Engineering faculty search where transportation is a potential sub-discipline within the department.</t>
+          <t>Moderate fit: broad Civil Engineering search where transportation is not explicitly prioritized in the snippet.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>Tenure-Track</t>
+          <t>Civil Engineering, Engineering Education</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Tuscaloosa, AL</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="inlineStr">
+          <t>Lake Charles, LA</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>Open until filled</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$76,000 per year</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Assistant Professor position in the Department of Civil, Construction and Environmental Engineering at the University of Alabama. | Research Topics: Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="L34" s="6" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/02ixzgls/Civil-Construction-and-Environmental-Engineering--Assistant-Professor</t>
-        </is>
-      </c>
-      <c r="M34" s="5" t="inlineStr">
-        <is>
-          <t>AcademicKeys</t>
+          <t>Assistant Professor position in Civil and Environmental Engineering at McNeese State University with a salary of $76,000 per year. | Research Topics: Civil Engineering, Engineering Education</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545361&amp;Title=Assistant%20Professor%20of%20Civil%20Engineering</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>HigherEdJobs</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -3600,85 +3600,85 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P34" s="5" t="inlineStr">
+      <c r="P34" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>33.2120822</v>
+        <v>30.1751363</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>-87.53967350000001</v>
+        <v>-93.2112786</v>
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>f80ad2336a210f82</t>
+          <t>bd292fb9f52ac2e9</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor of Civil, Construction and Environmental Engineering</t>
+          <t>Tenure-Track Faculty Positions in Transportation Engineering</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>University of Alabama</t>
+          <t>National Taiwan University</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil, Construction and Environmental Engineering</t>
+          <t>Department of Civil Engineering</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: Broad Civil, Construction, and Environmental Engineering Associate Professor opening without an explicitly specified sub-discipline.</t>
+          <t>Core match: seeks multiple tenure-track faculty positions specifically in the Transportation track within a Department of Civil Engineering.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Infrastructure</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>Tenured</t>
+          <t>Transportation Engineering, Mobility Systems, Transit Planning</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Tuscaloosa, AL</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
+          <t>Taipei, Taiwan</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>NT$83,720–137,370 monthly</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>The University of Alabama invites applications for an Associate Professor position in Civil, Construction, and Environmental Engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Infrastructure</t>
-        </is>
-      </c>
-      <c r="L35" s="6" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/w1r7nesq/Civil-Construction-and-Environmental-Engineering--Associate-Professor</t>
-        </is>
-      </c>
-      <c r="M35" s="5" t="inlineStr">
-        <is>
-          <t>AcademicKeys</t>
+          <t>The Department of Civil Engineering at National Taiwan University invites applications for multiple tenure-track faculty positions in Transportation Engineering. | Research Topics: Transportation Engineering, Mobility Systems, Transit Planning</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>https://jobs.chronicle.com/job/38034402/faculty-recruitment-announcement-department-of-civil-engineering-national-taiwan-university/</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -3691,382 +3691,18 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="P35" s="5" t="inlineStr">
+      <c r="P35" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>33.2120822</v>
+        <v>25.0375198</v>
       </c>
       <c r="R35" s="2" t="n">
-        <v>-87.53967350000001</v>
+        <v>121.5636796</v>
       </c>
       <c r="S35" s="2" t="inlineStr">
-        <is>
-          <t>1b5f034d56841a04</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Assistant Professor / Associate Professor (Tenure-Track) in Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Nanyang Technological University</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>School of Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Moderate fit: broad Civil and Environmental Engineering search where Transportation Engineering is a potential sub-discipline, though specific subfield requirements are not detailed in the snippet.</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>Tenure-Track</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>Singapore, Singapore</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
-          <t>Tenure-track Assistant or Associate Professor position in Civil and Environmental Engineering requiring an earned doctorate in civil engineering or a closely related discipline. | Research Topics: Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
-        </is>
-      </c>
-      <c r="L36" s="6" t="inlineStr">
-        <is>
-          <t>https://engineering.academickeys.com/job/dhzin0q4/Assistant-Professor--Associate-Professor-TenureTrack-in-Civil-and-Environmental-Engineering</t>
-        </is>
-      </c>
-      <c r="M36" s="5" t="inlineStr">
-        <is>
-          <t>AcademicKeys</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P36" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q36" s="2" t="n">
-        <v>1.2899175</v>
-      </c>
-      <c r="R36" s="2" t="n">
-        <v>103.8519072</v>
-      </c>
-      <c r="S36" s="2" t="inlineStr">
-        <is>
-          <t>3fa57c30724444e8</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Multiple Faculty Positions in Computer Science and Engineering</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Texas A&amp;M University</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Department of Computer Science and Engineering</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Moderate fit: open faculty search in Computer Science and Engineering without explicit specialization in transportation or mobility systems.</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>College Station, TX</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="K37" s="4" t="inlineStr">
-        <is>
-          <t>Texas A&amp;M University invites applications for multiple faculty positions in Computer Science and Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
-        </is>
-      </c>
-      <c r="L37" s="6" t="inlineStr">
-        <is>
-          <t>http://engineering.academickeys.com/job/rh7lvag4/CSE--TAMU-Multiple-Faculty-Positions</t>
-        </is>
-      </c>
-      <c r="M37" s="5" t="inlineStr">
-        <is>
-          <t>AcademicKeys</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O37" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P37" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q37" s="2" t="n">
-        <v>30.6187</v>
-      </c>
-      <c r="R37" s="2" t="n">
-        <v>-96.3365</v>
-      </c>
-      <c r="S37" s="2" t="inlineStr">
-        <is>
-          <t>7d5d844d65485b4b</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Assistant Professor of Civil Engineering</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>McNeese State University</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>Moderate fit: broad Civil Engineering search where transportation is not explicitly prioritized in the snippet.</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Civil Engineering, Engineering Education</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Lake Charles, LA</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>$76,000 per year</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr">
-        <is>
-          <t>Assistant Professor position in Civil and Environmental Engineering at McNeese State University with a salary of $76,000 per year. | Research Topics: Civil Engineering, Engineering Education</t>
-        </is>
-      </c>
-      <c r="L38" s="6" t="inlineStr">
-        <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545361&amp;Title=Assistant%20Professor%20of%20Civil%20Engineering</t>
-        </is>
-      </c>
-      <c r="M38" s="5" t="inlineStr">
-        <is>
-          <t>HigherEdJobs</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P38" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q38" s="2" t="n">
-        <v>30.1751363</v>
-      </c>
-      <c r="R38" s="2" t="n">
-        <v>-93.2112786</v>
-      </c>
-      <c r="S38" s="2" t="inlineStr">
-        <is>
-          <t>bd292fb9f52ac2e9</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Tenure-Track Faculty Positions in Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>National Taiwan University</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Department of Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>Core match: seeks multiple tenure-track faculty positions specifically in the Transportation track within a Department of Civil Engineering.</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>Transportation Engineering, Mobility Systems, Transit Planning</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>Tenure-Track</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Taipei, Taiwan</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>NT$83,720–137,370 monthly</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>The Department of Civil Engineering at National Taiwan University invites applications for multiple tenure-track faculty positions in Transportation Engineering. | Research Topics: Transportation Engineering, Mobility Systems, Transit Planning</t>
-        </is>
-      </c>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38034402/faculty-recruitment-announcement-department-of-civil-engineering-national-taiwan-university/</t>
-        </is>
-      </c>
-      <c r="M39" s="5" t="inlineStr">
-        <is>
-          <t>Chronicle</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O39" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P39" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q39" s="2" t="n">
-        <v>25.0375198</v>
-      </c>
-      <c r="R39" s="2" t="n">
-        <v>121.5636796</v>
-      </c>
-      <c r="S39" s="2" t="inlineStr">
         <is>
           <t>f056997ace2e1de7</t>
         </is>
@@ -4108,10 +3744,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand search queries to include Mobility and Public Transportation; update active listings to 46 positions
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -43,13 +43,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001F497D"/>
+      <b val="1"/>
+      <color rgb="00276A3C"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00276A3C"/>
+      <color rgb="001F497D"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -68,14 +68,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDF2F8"/>
-        <bgColor rgb="00EDF2F8"/>
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00EDF2F8"/>
+        <bgColor rgb="00EDF2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:S47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -505,7 +505,7 @@
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="83" customWidth="1" min="9" max="9"/>
-    <col width="47" customWidth="1" min="10" max="10"/>
+    <col width="96" customWidth="1" min="10" max="10"/>
     <col width="42" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
@@ -708,65 +708,65 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Civil, Construction and Environmental Engineering</t>
+          <t>Lecturer - Continuing Education</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>University of Alabama</t>
+          <t>City Colleges of Chicago</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Civil, Construction and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>6</v>
+          <t>Continuing Education</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Broad Civil, Construction and Environmental Engineering faculty search where transportation is a potential sub-discipline within the department.</t>
+          <t>Low fit: general continuing education lecturing position at a community college system without a focus on transportation engineering research or faculty track.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Engineering</t>
+          <t>Continuing Education, Community College Instruction, Adult Education</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Tuscaloosa, AL</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Competitive Salary</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Assistant Professor position in the Department of Civil, Construction and Environmental Engineering at the University of Alabama. | Research Topics: Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Engineering</t>
+          <t>This continuing education lecturer role provides instruction for adult learners within the City Colleges of Chicago system. | Research Topics: Continuing Education, Community College Instruction, Adult Education</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>https://engineering.academickeys.com/job/02ixzgls/Civil-Construction-and-Environmental-Engineering--Assistant-Professor</t>
+          <t>https://jobs.chronicle.com/job/37994648/lecturer-continuing-education/</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>AcademicKeys</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -785,59 +785,59 @@
         </is>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>33.2120822</v>
+        <v>32.898417</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>-87.53967350000001</v>
+        <v>-80.05262430000001</v>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>f80ad2336a210f82</t>
+          <t>aca94749a7e8bf9e</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Transportation Engineering</t>
+          <t>Professor / Associate Professor / Assistant Professor</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>South Dakota State University</t>
+          <t>The Hong Kong Polytechnic University</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>10</v>
+          <t>Department of Aeronautical and Aviation Engineering</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Core match: direct faculty position in Transportation Engineering aligning perfectly with the candidate's core field.</t>
+          <t>Low fit: position is in Aeronautical and Aviation Engineering, which falls outside the candidate's core transportation engineering and planning track.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Traffic Systems, Infrastructure Planning, Smart Mobility</t>
+          <t>Aeronautical Engineering, Aviation Engineering</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Brookings, SD</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -847,22 +847,22 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Assistant Professor position in Transportation Engineering requiring a Ph.D. in civil engineering or a closely related field to teach, advise, and conduct sponsored research. | Research Topics: Transportation Engineering, Traffic Systems, Infrastructure Planning, Smart Mobility</t>
+          <t>Faculty position in the Department of Aeronautical and Aviation Engineering at The Hong Kong Polytechnic University. | Research Topics: Aeronautical Engineering, Aviation Engineering</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>https://engineering.academickeys.com/job/m4lk5asr/Assistant-Professor-of-Transportation-Engineering</t>
+          <t>https://jobs.chronicle.com/job/38028368/professor-associate-professor-assistant-professor/</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>AcademicKeys</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -876,54 +876,54 @@
         </is>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>44.344449</v>
+        <v>22.3492361</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>-96.79823709999999</v>
+        <v>114.1857778</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>9b7d5de4753a514b</t>
+          <t>09d04da628fd08f9</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor of Civil Engineering (Transportation)</t>
+          <t>Assistant Professor of Teaching of Urban Planning</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Trine University</t>
+          <t>University of California, Los Angeles (UCLA)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n">
+          <t>Meyer and Renee Luskin School of Public Affairs, Department of Urban Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
         <v>8</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Strong match for a faculty position specifically dedicated to transportation engineering within a civil engineering program.</t>
+          <t>Strong interdisciplinary match for a faculty position in urban planning within the candidate's target department scope.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Civil Engineering Education, Intelligent Transportation Systems</t>
+          <t>Urban Planning, Teaching Mission, Mobility and Transportation Planning</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Angola, IN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -933,17 +933,17 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Based on qualifications</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>This is a faculty position seeking a transportation engineering specialist to teach undergraduate and graduate civil engineering courses and mentor students. | Research Topics: Transportation Engineering, Civil Engineering Education, Intelligent Transportation Systems</t>
+          <t>UCLA seeks an Assistant Professor of Teaching in Urban Planning to contribute primarily to the department's teaching mission. | Research Topics: Urban Planning, Teaching Mission, Mobility and Transportation Planning</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.chronicle.com/job/38028401/assistant-associate-professor-civil-engineering-transportation-/</t>
+          <t>https://jobs.chronicle.com/job/38020965/assistant-professor-of-teaching-of-urban-planning/</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -967,74 +967,74 @@
         </is>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>41.6311141</v>
+        <v>34.0536909</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>-85.0105982</v>
+        <v>-118.242766</v>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>9f9cc58aa59ccd96</t>
+          <t>fb7ba0794bd02172</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Urban Planning/Geography</t>
+          <t>Clinical Assistant Professor</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Loyola Marymount University</t>
+          <t>Georgia State University</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Department of Urban Planning</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>7</v>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match in urban planning and geography with potential focus on urban mobility and transit systems.</t>
+          <t>Low fit: the job snippet lacks specific department and topic details beyond a generic clinical assistant professor title at Georgia State University.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Urban Planning, Geography, Mobility Systems, Urban Analytics</t>
+          <t>Higher Education, Clinical Faculty, Not specified</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>$92,000</t>
+          <t>Competitive Salary</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Assistant Professor position in urban planning and geography requiring a terminal degree in a relevant field to teach and conduct research. | Research Topics: Urban Planning, Geography, Mobility Systems, Urban Analytics</t>
+          <t>This is a clinical assistant professor position at Georgia State University, but the specific academic discipline and research focus are not provided in the text. | Research Topics: Higher Education, Clinical Faculty, Not specified</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.chronicle.com/job/38031694/assistant-professor-of-urban-planning-geography/</t>
+          <t>https://jobs.chronicle.com/job/38022215/clinical-assistant-professor-non-tenure-tack/</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1058,44 +1058,44 @@
         </is>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>33.9687824</v>
+        <v>33.7535889</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>-118.4182021</v>
+        <v>-84.3854209</v>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>c13b0c3f0cf09a9e</t>
+          <t>f39f14cbaaf9d6f7</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Urban Economics</t>
+          <t>Assistant Professor of Public Policy (Market-Based Solutions to Societal Challenges)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Harvard University</t>
+          <t>University of Wisconsin-Madison</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Department of Economics / Graduate School of Design</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>5</v>
+          <t>Department of Public Policy / La Follette School of Public Affairs</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: urban economics position focusing on economic analysis rather than core transportation engineering and travel behavior.</t>
+          <t>Low fit: public policy position focused on market-based solutions rather than core transportation engineering or mobility systems.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Urban Economics, Spatial Economics, Urban Analytics, Real Estate and Housing</t>
+          <t>Public Policy, Market-Based Solutions, Societal Challenges</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Cambridge, MA</t>
+          <t>Madison, WI</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1115,17 +1115,17 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>$165,000 - $185,000</t>
+          <t>Competitive Salary</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track faculty role in urban economics requiring a Ph.D. in economics, public policy, or a closely related field with a focus on urban systems. | Research Topics: Urban Economics, Spatial Economics, Urban Analytics, Real Estate and Housing</t>
+          <t>An assistant professor position in public policy focusing on market-based solutions to societal challenges requiring a Ph.D. or equivalent. | Research Topics: Public Policy, Market-Based Solutions, Societal Challenges</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.chronicle.com/job/38032116/assistant-professor-urban-economics-/</t>
+          <t>https://jobs.chronicle.com/job/38008254/assistant-professor-of-public-policy-market-based-solutions-to-societal-challenges-/</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -1149,74 +1149,74 @@
         </is>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>42.3657432</v>
+        <v>43.0802745</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>-71.12221390000001</v>
+        <v>-89.43095870000001</v>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>93251b0fa8170f49</t>
+          <t>51857534b7308d30</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Adjunct Faculty - Transportation Engineering</t>
+          <t>Assistant Professor in Industrial Engineering</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Morgan State University</t>
+          <t>California Polytechnic State University - San Luis Obispo</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Civil and Environmental Engineering</t>
+          <t>Industrial and Manufacturing Engineering (IME) Department</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Core match: directly seeks faculty expertise in Transportation Engineering.</t>
+          <t>Moderate fit: An Industrial Engineering faculty position at Cal Poly, which falls into a target department but lacks specific mention of transportation or mobility systems in the brief snippet.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Transit Planning, Traffic Systems</t>
+          <t>Industrial Engineering, Systems Engineering, Manufacturing Engineering</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Non-Tenure Track</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Baltimore, MD</t>
+          <t>San Luis Obispo, CA</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Competitive Salary</t>
+          <t>$106,000 - $117,000 per year</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>The role seeks an adjunct faculty member to teach transportation engineering courses within the civil and environmental engineering department, requiring a relevant graduate degree. | Research Topics: Transportation Engineering, Transit Planning, Traffic Systems</t>
+          <t>Full-time Assistant Professor in Industrial Engineering at California Polytechnic State University starting August 12th. | Research Topics: Industrial Engineering, Systems Engineering, Manufacturing Engineering</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.chronicle.com/job/37974518/adjunct-faculty-transportation-engineering/</t>
+          <t>https://jobs.chronicle.com/job/38018328/assistant-professor-industrial-engineering/</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1240,74 +1240,74 @@
         </is>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>39.3446663</v>
+        <v>35.3074623</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>-76.5836094</v>
+        <v>-120.6646483</v>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>3df6fb24b156d70b</t>
+          <t>78cbe3317d3f9c95</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Advanced Transportation Technology Instructor, Part-time Adjunct</t>
+          <t>Assistant Professor in Urban and Regional Planning</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Kern Community College District</t>
+          <t>Louisiana State University New Orleans</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Advanced Transportation Technology</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>5</v>
+          <t>Planning and Urban Studies</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>7</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: community college instructor position in advanced transportation technology, but lacks tenure-track research focus.</t>
+          <t>Strong interdisciplinary match for an Assistant Professor position in Urban and Regional Planning, which aligns with the candidate's mobility and urban planning target track.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Advanced Transportation Technology, Vehicle Technologies, Transportation Education</t>
+          <t>Urban and Regional Planning, Urban Studies, Mobility Systems</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Non-Tenure Track</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>New Orleans, LA</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>$65.00 Hourly</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Part-time adjunct instructor role teaching advanced transportation technology courses at a community college district. | Research Topics: Advanced Transportation Technology, Vehicle Technologies, Transportation Education</t>
+          <t>Louisiana State University New Orleans invites applications for a tenure-track Assistant Professor position in Urban and Regional Planning. | Research Topics: Urban and Regional Planning, Urban Studies, Mobility Systems</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.chronicle.com/job/38026829/advanced-transportation-technology-instructor-part-time-adjunct/</t>
+          <t>https://jobs.chronicle.com/job/38025681/assistant-professor-planning-and-urban-studies-/</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1331,44 +1331,44 @@
         </is>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>37.8719</v>
+        <v>29.9911944</v>
       </c>
       <c r="R9" s="2" t="n">
-        <v>-122.2585</v>
+        <v>-90.0835067</v>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>36f117729bac62c9</t>
+          <t>f373f0209d1c2577</t>
         </is>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate/Full Professor, Transportation Engineering and Systems</t>
+          <t>Assistant Professor of Technology and Social Change</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>University of Cincinnati</t>
+          <t>The Ohio State University</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil and Architectural Engineering and Construction Management</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>10</v>
+          <t>Department of Sociology</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Core match: explicitly seeks a faculty member in Transportation Engineering and Systems within a Civil Engineering department.</t>
+          <t>Low fit: position is in the Department of Sociology focusing on technology and social change rather than transportation engineering or mobility.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Transportation Systems, Transit Planning, Mobility Systems</t>
+          <t>Technology and Social Change, Sociology of Technology</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1378,37 +1378,37 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Cincinnati, OH</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Commensurate with education and experience</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>The Department of Civil and Architectural Engineering and Construction Management at the University of Cincinnati is seeking an open-rank faculty member specializing in transportation engineering and systems. | Research Topics: Transportation Engineering, Transportation Systems, Transit Planning, Mobility Systems</t>
+          <t>The Department of Sociology at The Ohio State University seeks a tenure-track Assistant Professor in Technology and Social Change. | Research Topics: Technology and Social Change, Sociology of Technology</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-transportation-engineering-and-systems-at-university-of-cincinnati-4416744025</t>
+          <t>https://jobs.chronicle.com/job/38029743/assistant-professor-of-technology-and-social-change/</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1422,54 +1422,54 @@
         </is>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>39.1318888</v>
+        <v>40.0067</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>-84.51578309999999</v>
+        <v>-83.0305</v>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>6aa8ab000bc6f6c0</t>
+          <t>66008413c6bf1b19</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor of Civil, Architectural and Environmental Engineering</t>
+          <t>Full/Associate/Assistant Professor in Modern Civil Engineering</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Missouri University of Science and Technology</t>
+          <t>University of Macau</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Civil, Architectural and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>6</v>
+          <t>Faculty of Engineering</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: a broad Civil, Architectural and Environmental Engineering department search that may include transportation, though the specific sub-discipline focus in the provided snippet is unspecified.</t>
+          <t>Moderate fit: broad modern civil engineering position at the University of Macau in Macau, but outside the target geographic scope (Mainland China / SAR region not in preferred US/EU/East Asia target list) and lacking specific focus on transportation.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Architectural Engineering, Environmental Engineering</t>
+          <t>Modern Civil Engineering, Infrastructure, Engineering Education</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Rolla, MO</t>
+          <t>Macau</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1479,27 +1479,27 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Commensurate with the applicants’ academic qualification and relevant professional experience</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>The position seeks an Assistant or Associate Professor in the Department of Civil, Architectural and Environmental Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Civil Engineering, Architectural Engineering, Environmental Engineering</t>
+          <t>The University of Macau invites applications for a faculty position in Modern Civil Engineering within the Faculty of Engineering. | Research Topics: Modern Civil Engineering, Infrastructure, Engineering Education</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-associate-professor-civil-architectural-and-environmental-engineering-%2300096512-at-missouri-university-of-science-and-technology-4442271248</t>
+          <t>https://jobs.chronicle.com/job/38020589/full-associate-assistant-professor-in-modern-civil-engineering/</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1513,44 +1513,44 @@
         </is>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>37.9532435</v>
+        <v>22.1757605</v>
       </c>
       <c r="R11" s="2" t="n">
-        <v>-91.7742667</v>
+        <v>113.5514142</v>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>4fad8c46021c1243</t>
+          <t>f5ea2aadd95a9b14</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Transportation Policy</t>
+          <t>Tenure-Track Assistant Professor of Statistics</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Hunter College</t>
+          <t>Haverford College</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Department of Urban Policy and Planning, School of Arts and Sciences</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>8</v>
+          <t>Department of Mathematics and Statistics</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match in an Urban Policy and Planning department specifically seeking expertise in transportation policy, accessibility, and equity.</t>
+          <t>Low fit: position is in Statistics rather than Transportation Engineering or Mobility Systems.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Transportation Policy, Transit Accessibility, Transportation Equity, Community-Engaged Research</t>
+          <t>Statistics, Data Analysis, Mathematics</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1560,37 +1560,37 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Haverford, PA</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Open until filled (Review begins Oct. 1, 2025)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>$77,092 - $91,922 (plus scheduled increases)</t>
+          <t>Competitive Salary</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Hunter College seeks a tenure-track Assistant Professor in transportation policy requiring a Ph.D. in policy, planning, or a related field to teach applied policy research and develop a robust research agenda. | Research Topics: Transportation Policy, Transit Accessibility, Transportation Equity, Community-Engaged Research</t>
+          <t>Haverford College seeks a tenure-track Assistant Professor of Statistics to begin in fall 2027 within the Department of Mathematics and Statistics. | Research Topics: Statistics, Data Analysis, Mathematics</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-urban-policy-and-planning-dept-school-of-arts-and-sciences-hunter-college-at-hunter-college-4438624127</t>
+          <t>https://jobs.chronicle.com/job/38017766/tenure-track-assistant-professor-of-statistics/</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1604,89 +1604,89 @@
         </is>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>40.7683107</v>
+        <v>40.0071506</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>-73.964406</v>
+        <v>-75.3069423</v>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>e4e18ed629103a27</t>
+          <t>139bc27f2f7867a0</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Research Assistant Professor</t>
+          <t>Assistant Professor of Operations Management</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>University of Houston</t>
+          <t>University of Illinois - Chicago</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Information Science Technology (CYBER-CARE Consortium)</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>6</v>
+          <t>Information and Decision Sciences (IDS) Department</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: the role is a Research Assistant Professor position in transportation engineering, but heavily emphasizes cybersecurity and connected/automated vehicles rather than the candidate's core focus on travel behavior and transit planning.</t>
+          <t>Low fit: position is in Supply Chain and Operations Management within a business/IDS department rather than transportation engineering or urban planning.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Connected and Automated Vehicle Cybersecurity, Transportation Data Security, Advanced Traffic Management Systems, Intelligent Transportation Systems</t>
+          <t>Operations Management, Supply Chain Management</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Non-Tenure Track</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Commensurate with experience</t>
+          <t>DOE</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>The University of Houston seeks a non-tenure track Research Assistant Professor for the CYBER-CARE consortium to conduct research on transportation cybersecurity and AI applications, requiring a doctoral degree in Transportation Engineering or a closely related field. | Research Topics: Connected and Automated Vehicle Cybersecurity, Transportation Data Security, Advanced Traffic Management Systems, Intelligent Transportation Systems</t>
+          <t>The Information and Decision Sciences department invites applications for a tenure-track assistant professor position in Operations Management starting in the 2027-2028 academic year. | Research Topics: Operations Management, Supply Chain Management</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/research-assistant-professor-cyber-care-consortium-at-university-of-houston-4404319276</t>
+          <t>https://jobs.chronicle.com/job/38035040/assistant-professor-ids-supply-chain-and-operations-management-/</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P13" s="3" t="inlineStr">
@@ -1695,44 +1695,44 @@
         </is>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>29.7207902</v>
+        <v>41.8748613</v>
       </c>
       <c r="R13" s="2" t="n">
-        <v>-95.34406269999999</v>
+        <v>-87.6519866</v>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>c6ee2c0289357949</t>
+          <t>c1e8cde424bc7afa</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Tenure-Track Assistant/Associate Professor of Air Transportation Systems</t>
+          <t>Tenure-track Assistant Professor of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Embry-Riddle Aeronautical University</t>
+          <t>University of Tennessee, Knoxville</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>School of Graduate Studies in the College of Aviation</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>4</v>
+          <t>Department of Industrial and Systems Engineering</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Moderate-low fit: the position focuses specifically on aviation and aerospace systems (air transportation, advanced air mobility, UAS) rather than surface transportation engineering or mobility.</t>
+          <t>Moderate fit: Assistant Professor position in Industrial and Systems Engineering which can align with mobility systems, though the snippet lacks specific details.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Air Transportation Systems, Advanced Air Mobility, UAS Traffic Management, Machine Learning/AI in Aviation</t>
+          <t>Industrial Engineering, Systems Engineering, Mobility Systems</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1742,42 +1742,42 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Daytona Beach, FL</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Review begins immediately; Priority given to applications received by 2026-08-31</t>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Competitive Salary</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>This tenure-track faculty position requires a doctorate in air transportation systems, advanced air mobility, or a related area to teach graduate courses and conduct AI/machine learning research in aviation. | Research Topics: Air Transportation Systems, Advanced Air Mobility, UAS Traffic Management, Machine Learning/AI in Aviation</t>
+          <t>The University of Tennessee, Knoxville is seeking three tenure-track Assistant Professors in the Department of Industrial and Systems Engineering. | Research Topics: Industrial Engineering, Systems Engineering, Mobility Systems</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/tenure-track-faculty-position-with-a-focus-on-air-transportation-systems-daytona-beach-campus-at-embry-riddle-aeronautical-university-4434897662</t>
+          <t>https://jobs.chronicle.com/job/38032334/tenure-track-assistant-professor-of-industrial-and-systems-engineering-fall-2027-1-3-/</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P14" s="3" t="inlineStr">
@@ -1786,44 +1786,44 @@
         </is>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>33.8082375</v>
+        <v>35.9516352</v>
       </c>
       <c r="R14" s="2" t="n">
-        <v>-118.1344224</v>
+        <v>-83.9308819</v>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>b3c177958e0ab7a7</t>
+          <t>a40790e93b28a33d</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor / Associate Professor (Tenure-Track) in Civil and Environmental Engineering</t>
+          <t>Assistant Professor of Civil, Construction and Environmental Engineering</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Nanyang Technological University</t>
+          <t>University of Alabama</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>School of Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>5</v>
+          <t>Civil, Construction and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: broad Civil and Environmental Engineering search where Transportation Engineering is a potential sub-discipline, though specific subfield requirements are not detailed in the snippet.</t>
+          <t>Broad Civil, Construction and Environmental Engineering faculty search where transportation is a potential sub-discipline within the department.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
+          <t>Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Engineering</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Singapore, Singapore</t>
+          <t>Tuscaloosa, AL</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1848,12 +1848,12 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Tenure-track Assistant or Associate Professor position in Civil and Environmental Engineering requiring an earned doctorate in civil engineering or a closely related discipline. | Research Topics: Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
+          <t>Assistant Professor position in the Department of Civil, Construction and Environmental Engineering at the University of Alabama. | Research Topics: Civil Engineering, Construction Engineering, Environmental Engineering, Transportation Engineering</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>https://engineering.academickeys.com/job/dhzin0q4/Assistant-Professor--Associate-Professor-TenureTrack-in-Civil-and-Environmental-Engineering</t>
+          <t>https://engineering.academickeys.com/job/02ixzgls/Civil-Construction-and-Environmental-Engineering--Assistant-Professor</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -1877,44 +1877,44 @@
         </is>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>1.2899175</v>
+        <v>33.2120822</v>
       </c>
       <c r="R15" s="2" t="n">
-        <v>103.8519072</v>
+        <v>-87.53967350000001</v>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>3fa57c30724444e8</t>
+          <t>f80ad2336a210f82</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Assistant / Associate / Full Professor of Mechanical Engineering</t>
+          <t>Assistant Professor of Transportation Engineering</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Auburn University</t>
+          <t>South Dakota State University</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Department of Mechanical Engineering</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>3</v>
+          <t>Department of Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>10</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Low fit: position is in Mechanical Engineering and lacks description details, which does not align with the candidate's transportation engineering and planning profile.</t>
+          <t>Core match: direct faculty position in Transportation Engineering aligning perfectly with the candidate's core field.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
+          <t>Transportation Engineering, Traffic Systems, Infrastructure Planning, Smart Mobility</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1924,27 +1924,27 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Auburn, AL</t>
+          <t>Brookings, SD</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>An open-rank faculty position in mechanical engineering requiring a Ph.D. in mechanical engineering or a closely related field. | Research Topics: Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
+          <t>Assistant Professor position in Transportation Engineering requiring a Ph.D. in civil engineering or a closely related field to teach, advise, and conduct sponsored research. | Research Topics: Transportation Engineering, Traffic Systems, Infrastructure Planning, Smart Mobility</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>https://engineering.academickeys.com/job/f320isty/AssistantAssociateFull-Professor</t>
+          <t>https://engineering.academickeys.com/job/m4lk5asr/Assistant-Professor-of-Transportation-Engineering</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1968,44 +1968,44 @@
         </is>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>32.5919529</v>
+        <v>44.344449</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>-85.4959775</v>
+        <v>-96.79823709999999</v>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>c08698a4bf95171b</t>
+          <t>9b7d5de4753a514b</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Assistant / Associate Professor of Industrial and Systems Engineering</t>
+          <t>Assistant/Associate Professor of Civil Engineering (Transportation)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>University of Washington</t>
+          <t>Trine University</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Industrial and Systems Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match: industrial and systems engineering position in a target department, though specific mobility focus depends on the full department scope.</t>
+          <t>Strong match for a faculty position specifically dedicated to transportation engineering within a civil engineering program.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
+          <t>Transportation Engineering, Civil Engineering Education, Intelligent Transportation Systems</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -2015,37 +2015,37 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Angola, IN</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Based on qualifications</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Assistant or Associate Professor position in Industrial and Systems Engineering requiring a Ph.D. in a relevant engineering or analytical discipline. | Research Topics: Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
+          <t>This is a faculty position seeking a transportation engineering specialist to teach undergraduate and graduate civil engineering courses and mentor students. | Research Topics: Transportation Engineering, Civil Engineering Education, Intelligent Transportation Systems</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>https://engineering.academickeys.com/job/g4m97a60/AssistantAssociate-Professor-Industrial-and-Systems-Engineering-Systems-Engineering-Focus</t>
+          <t>https://jobs.chronicle.com/job/38028401/assistant-associate-professor-civil-engineering-transportation-/</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>AcademicKeys</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -2059,54 +2059,54 @@
         </is>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>47.6553</v>
+        <v>41.6311141</v>
       </c>
       <c r="R17" s="2" t="n">
-        <v>-122.3035</v>
+        <v>-85.0105982</v>
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>9d5682cf4dbca334</t>
+          <t>9f9cc58aa59ccd96</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Professor &amp; Department Chair</t>
+          <t>Assistant Professor of Urban Planning/Geography</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>University of Pittsburgh</t>
+          <t>Loyola Marymount University</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>3</v>
+          <t>Department of Urban Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>7</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Low fit: departmental leadership position for a broad Civil and Environmental Engineering department rather than a dedicated transportation research faculty role.</t>
+          <t>Strong interdisciplinary match in urban planning and geography with potential focus on urban mobility and transit systems.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
+          <t>Urban Planning, Geography, Mobility Systems, Urban Analytics</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Tenured</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -2116,27 +2116,27 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$92,000</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Strictly 1 concise sentence summarizing the primary focus of the role and minimum degree qualification. | Research Topics: Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
+          <t>Assistant Professor position in urban planning and geography requiring a terminal degree in a relevant field to teach and conduct research. | Research Topics: Urban Planning, Geography, Mobility Systems, Urban Analytics</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>http://engineering.academickeys.com/job/vhlo0w6p/Professor--Department-Chair--Electrical-and-Computer-Engineering</t>
+          <t>https://jobs.chronicle.com/job/38031694/assistant-professor-of-urban-planning-geography/</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>AcademicKeys</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -2150,84 +2150,84 @@
         </is>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>40.444153</v>
+        <v>33.9687824</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>-79.962461</v>
+        <v>-118.4182021</v>
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>17acd4b4e7207871</t>
+          <t>c13b0c3f0cf09a9e</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Lecturer in Discipline or Senior Lecturer in Discipline</t>
+          <t>Assistant Professor of Urban Economics</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Columbia University</t>
+          <t>Harvard University</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>6</v>
+          <t>Department of Economics / Graduate School of Design</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: general lecturer position at Columbia University in an unspecified discipline, requiring further text details to confirm a transportation focus.</t>
+          <t>Moderate fit: urban economics position focusing on economic analysis rather than core transportation engineering and travel behavior.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Higher Education, Instruction, Academic Teaching</t>
+          <t>Urban Economics, Spatial Economics, Urban Analytics, Real Estate and Housing</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Non-Tenure Track</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Cambridge, MA</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$165,000 - $185,000</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>This is a faculty teaching role at Columbia University, though the specific academic department and subject focus are missing from the current snippet. | Research Topics: Higher Education, Instruction, Academic Teaching</t>
+          <t>This is a tenure-track faculty role in urban economics requiring a Ph.D. in economics, public policy, or a closely related field with a focus on urban systems. | Research Topics: Urban Economics, Spatial Economics, Urban Analytics, Real Estate and Housing</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>http://engineering.academickeys.com/job/arsy3jqh/Open-Rank-Lecturer-in-Discipline-or-Senior-Lecturer-in-Discipline</t>
+          <t>https://jobs.chronicle.com/job/38032116/assistant-professor-urban-economics-/</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>AcademicKeys</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -2241,84 +2241,84 @@
         </is>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>40.8077507</v>
+        <v>42.3657432</v>
       </c>
       <c r="R19" s="2" t="n">
-        <v>-73.9624901</v>
+        <v>-71.12221390000001</v>
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>f11b4a4e74422ae3</t>
+          <t>93251b0fa8170f49</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor of Civil Engineering</t>
+          <t>Adjunct Faculty - Transportation Engineering</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Cedarville University</t>
+          <t>Morgan State University</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil Engineering</t>
+          <t>Civil and Environmental Engineering</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: broad Civil Engineering search where transportation may be acceptable, but lacks a dedicated job description snippet for precise evaluation.</t>
+          <t>Core match: directly seeks faculty expertise in Transportation Engineering.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
+          <t>Transportation Engineering, Transit Planning, Traffic Systems</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Cedarville, OH</t>
+          <t>Baltimore, MD</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Competitive Salary</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>A faculty position in civil engineering requiring a Ph.D. to teach undergraduate courses and engage in scholarly activity. | Research Topics: Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
+          <t>The role seeks an adjunct faculty member to teach transportation engineering courses within the civil and environmental engineering department, requiring a relevant graduate degree. | Research Topics: Transportation Engineering, Transit Planning, Traffic Systems</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179544290&amp;Title=Assistant%2FAssociate%20Professor%20of%20Civil%20Engineering</t>
+          <t>https://jobs.chronicle.com/job/37974518/adjunct-faculty-transportation-engineering/</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>HigherEdJobs</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -2332,54 +2332,54 @@
         </is>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>39.7540491</v>
+        <v>39.3446663</v>
       </c>
       <c r="R20" s="2" t="n">
-        <v>-83.8170518</v>
+        <v>-76.5836094</v>
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>751c7406865a2787</t>
+          <t>3df6fb24b156d70b</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Information and Decision Sciences (Supply Chain &amp; Operations Management)</t>
+          <t>Advanced Transportation Technology Instructor, Part-time Adjunct</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>University of Illinois Chicago</t>
+          <t>Kern Community College District</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Information and Decision Sciences (IDS)</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>3</v>
+          <t>Advanced Transportation Technology</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Low fit: position is in Supply Chain and Operations Management within a business school, which falls outside the candidate's core transportation engineering and mobility systems profile.</t>
+          <t>Moderate fit: community college instructor position in advanced transportation technology, but lacks tenure-track research focus.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Operations Management, Decision Sciences</t>
+          <t>Advanced Transportation Technology, Vehicle Technologies, Transportation Education</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>California</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -2389,27 +2389,27 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$65.00 Hourly</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track Assistant Professor role in Supply Chain and Operations Management requiring a Ph.D. in a relevant business or analytical discipline. | Research Topics: Supply Chain Management, Operations Management, Decision Sciences</t>
+          <t>Part-time adjunct instructor role teaching advanced transportation technology courses at a community college district. | Research Topics: Advanced Transportation Technology, Vehicle Technologies, Transportation Education</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179552436&amp;Title=Assistant%20Professor%20%2D%20IDS%20%28Supply%20Chain%20%26%20Operations%20Management%29</t>
+          <t>https://jobs.chronicle.com/job/38026829/advanced-transportation-technology-instructor-part-time-adjunct/</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>HigherEdJobs</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -2423,44 +2423,44 @@
         </is>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>41.8748613</v>
+        <v>37.8719</v>
       </c>
       <c r="R21" s="2" t="n">
-        <v>-87.6519866</v>
+        <v>-122.2585</v>
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>77e0632bd4e74eae</t>
+          <t>36f117729bac62c9</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Professor, Associate Professor, or Assistant Professor of Industrial and Systems Engineering</t>
+          <t>Assistant/Associate/Full Professor, Transportation Engineering and Systems</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Auburn University</t>
+          <t>University of Cincinnati</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial and Systems Engineering</t>
+          <t>Department of Civil and Architectural Engineering and Construction Management</t>
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: Industrial and Systems Engineering faculty position at Auburn University, but the job description text was missing to confirm a specific focus on mobility systems.</t>
+          <t>Core match: explicitly seeks a faculty member in Transportation Engineering and Systems within a Civil Engineering department.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Industrial Engineering, Systems Engineering, Operations Research</t>
+          <t>Transportation Engineering, Transportation Systems, Transit Planning, Mobility Systems</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Auburn, AL</t>
+          <t>Cincinnati, OH</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -2480,27 +2480,27 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>$80,000 - $180,000 per year</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Open-rank faculty position in Industrial and Systems Engineering requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Systems Engineering, Operations Research</t>
+          <t>The Department of Civil and Architectural Engineering and Construction Management at the University of Cincinnati is seeking an open-rank faculty member specializing in transportation engineering and systems. | Research Topics: Transportation Engineering, Transportation Systems, Transit Planning, Mobility Systems</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179548357&amp;Title=Professor%2C%20Associate%20Professor%2C%20Assistant%20Professor%20%2D%20Industrial%20and%20Systems%20Engineering</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-transportation-engineering-and-systems-at-university-of-cincinnati-4416744025</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>HigherEdJobs</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -2514,44 +2514,44 @@
         </is>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>32.5919529</v>
+        <v>39.1318888</v>
       </c>
       <c r="R22" s="2" t="n">
-        <v>-85.4959775</v>
+        <v>-84.51578309999999</v>
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>d0f23a527bf71c22</t>
+          <t>6aa8ab000bc6f6c0</t>
         </is>
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Tenure-Track Assistant Professor of Industrial and Systems Engineering</t>
+          <t>Assistant/Associate Professor of Civil, Architectural and Environmental Engineering</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>University of Tennessee, Knoxville</t>
+          <t>Missouri University of Science and Technology</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial and Systems Engineering</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>7</v>
+          <t>Civil, Architectural and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match in Industrial and Systems Engineering with a focus on mobility systems aligned with the candidate's target departments.</t>
+          <t>Moderate fit: a broad Civil, Architectural and Environmental Engineering department search that may include transportation, though the specific sub-discipline focus in the provided snippet is unspecified.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Industrial Engineering, Mobility Systems, Systems Engineering</t>
+          <t>Civil Engineering, Architectural Engineering, Environmental Engineering</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Knoxville, TN</t>
+          <t>Rolla, MO</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -2576,22 +2576,22 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Tenure-track Assistant Professor position in Industrial and Systems Engineering focusing on mobility systems, requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Mobility Systems, Systems Engineering</t>
+          <t>The position seeks an Assistant or Associate Professor in the Department of Civil, Architectural and Environmental Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Civil Engineering, Architectural Engineering, Environmental Engineering</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545449&amp;Title=Tenure%2DTrack%20Assistant%20Professor%20of%20Industrial%20and%20Systems%20Engineering%2C%20Fall%202027%20%281%2F3%29</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-associate-professor-civil-architectural-and-environmental-engineering-%2300096512-at-missouri-university-of-science-and-technology-4442271248</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>HigherEdJobs</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -2605,84 +2605,84 @@
         </is>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>35.9516352</v>
+        <v>37.9532435</v>
       </c>
       <c r="R23" s="2" t="n">
-        <v>-83.9308819</v>
+        <v>-91.7742667</v>
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>ecd34777430b7c8d</t>
+          <t>4fad8c46021c1243</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Teaching Assistant Professor</t>
+          <t>Assistant Professor in Transportation Policy</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>Hunter College</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Department of Urban Policy and Planning, School of Arts and Sciences</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: Broad Civil Engineering faculty search where transportation is only one of multiple acceptable sub-disciplines.</t>
+          <t>Strong interdisciplinary match in an Urban Policy and Planning department specifically seeking expertise in transportation policy, accessibility, and equity.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering Education, Transportation Engineering</t>
+          <t>Transportation Policy, Transit Accessibility, Transportation Equity, Community-Engaged Research</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Non-Tenure Track</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Open until filled (Review begins Oct. 1, 2025)</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$77,092 - $91,922 (plus scheduled increases)</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>A teaching-focused assistant professor position in civil engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Civil Engineering Education, Transportation Engineering</t>
+          <t>Hunter College seeks a tenure-track Assistant Professor in transportation policy requiring a Ph.D. in policy, planning, or a related field to teach applied policy research and develop a robust research agenda. | Research Topics: Transportation Policy, Transit Accessibility, Transportation Equity, Community-Engaged Research</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179541925&amp;Title=Teaching%20Assistant%20Professor</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-urban-policy-and-planning-dept-school-of-arts-and-sciences-hunter-college-at-hunter-college-4438624127</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>HigherEdJobs</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -2696,44 +2696,44 @@
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>36.0970389</v>
+        <v>40.7683107</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>-94.1703322</v>
+        <v>-73.964406</v>
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>8b28f5b58e7e3607</t>
+          <t>e4e18ed629103a27</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Teaching</t>
+          <t>Research Assistant Professor</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Florida Atlantic University</t>
+          <t>University of Houston</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil, Environmental &amp; Geomatics Engineering</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>5</v>
+          <t>Information Science Technology (CYBER-CARE Consortium)</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: it is a Civil Engineering teaching position in a department with transportation research centers, but requires teaching structural analysis and design-related classes alongside a P.E. license.</t>
+          <t>Moderate fit: the role is a Research Assistant Professor position in transportation engineering, but heavily emphasizes cybersecurity and connected/automated vehicles rather than the candidate's core focus on travel behavior and transit planning.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+          <t>Connected and Automated Vehicle Cybersecurity, Transportation Data Security, Advanced Traffic Management Systems, Intelligent Transportation Systems</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Boca Raton, FL</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -2753,17 +2753,17 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Commensurate with Experience</t>
+          <t>Commensurate with experience</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>This is a non-tenure-track Assistant Teaching Professor position in civil engineering requiring a Ph.D. and P.E. license to teach undergraduate and graduate courses including structural analysis and design. | Research Topics: Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+          <t>The University of Houston seeks a non-tenure track Research Assistant Professor for the CYBER-CARE consortium to conduct research on transportation cybersecurity and AI applications, requiring a doctoral degree in Transportation Engineering or a closely related field. | Research Topics: Connected and Automated Vehicle Cybersecurity, Transportation Data Security, Advanced Traffic Management Systems, Intelligent Transportation Systems</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-teaching-at-florida-atlantic-university-4414964381</t>
+          <t>https://www.linkedin.com/jobs/view/research-assistant-professor-cyber-care-consortium-at-university-of-houston-4404319276</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
@@ -2773,58 +2773,58 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>26.1194058</v>
+        <v>29.7207902</v>
       </c>
       <c r="R25" s="2" t="n">
-        <v>-80.14167999999999</v>
+        <v>-95.34406269999999</v>
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>7bdaa996cf64d1f6</t>
+          <t>c6ee2c0289357949</t>
         </is>
       </c>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Assistant or Associate Professor in Supply Chain Management</t>
+          <t>Tenure-Track Assistant/Associate Professor of Air Transportation Systems</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>Embry-Riddle Aeronautical University</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>J.B. Hunt Transport Department of Supply Chain Management</t>
+          <t>School of Graduate Studies in the College of Aviation</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Low fit: this is a faculty position in Supply Chain Management within a Business School rather than Transportation Engineering.</t>
+          <t>Moderate-low fit: the position focuses specifically on aviation and aerospace systems (air transportation, advanced air mobility, UAS) rather than surface transportation engineering or mobility.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Logistics, Operations Research</t>
+          <t>Air Transportation Systems, Advanced Air Mobility, UAS Traffic Management, Machine Learning/AI in Aviation</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -2834,12 +2834,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
+          <t>Daytona Beach, FL</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>Review begins immediately; Priority given to applications received by 2026-08-31</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2849,12 +2849,12 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track Assistant or Associate Professor position in Supply Chain Management requiring a strong research record in leading peer-reviewed journals. | Research Topics: Supply Chain Management, Logistics, Operations Research</t>
+          <t>This tenure-track faculty position requires a doctorate in air transportation systems, advanced air mobility, or a related area to teach graduate courses and conduct AI/machine learning research in aviation. | Research Topics: Air Transportation Systems, Advanced Air Mobility, UAS Traffic Management, Machine Learning/AI in Aviation</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-or-associate-professor-open-rank-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460111187</t>
+          <t>https://www.linkedin.com/jobs/view/tenure-track-faculty-position-with-a-focus-on-air-transportation-systems-daytona-beach-campus-at-embry-riddle-aeronautical-university-4434897662</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
@@ -2864,58 +2864,58 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
       <c r="P26" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>36.0625843</v>
+        <v>33.8082375</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>-94.1574328</v>
+        <v>-118.1344224</v>
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>c16a694d5f7f68d4</t>
+          <t>b3c177958e0ab7a7</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Aerospace Engineering</t>
+          <t>Assistant Professor / Associate Professor (Tenure-Track) in Civil and Environmental Engineering</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>The University of Kansas</t>
+          <t>Nanyang Technological University</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Department of Aerospace Engineering</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>3</v>
+          <t>School of Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>The position is specifically for Aerospace Engineering focusing on aircraft and space systems, where the candidate's core transportation engineering expertise is not the primary requirement.</t>
+          <t>Moderate fit: broad Civil and Environmental Engineering search where Transportation Engineering is a potential sub-discipline, though specific subfield requirements are not detailed in the snippet.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+          <t>Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -2925,37 +2925,37 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Lawrence, KS</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track faculty position in Aerospace Engineering requiring a doctorate in Aerospace Engineering or a closely related field, focusing on aviation and space-related research. | Research Topics: Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+          <t>Tenure-track Assistant or Associate Professor position in Civil and Environmental Engineering requiring an earned doctorate in civil engineering or a closely related discipline. | Research Topics: Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-aerospace-engineering-at-the-university-of-kansas-4460398978</t>
+          <t>https://engineering.academickeys.com/job/dhzin0q4/Assistant-Professor--Associate-Professor-TenureTrack-in-Civil-and-Environmental-Engineering</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
@@ -2969,44 +2969,44 @@
         </is>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>39.0559267</v>
+        <v>1.2899175</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>-94.6090332</v>
+        <v>103.8519072</v>
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>4a53cfad86712a72</t>
+          <t>3fa57c30724444e8</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate/Full Professor in Industrial and Systems Engineering</t>
+          <t>Assistant / Associate / Full Professor of Mechanical Engineering</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>University of Florida</t>
+          <t>Auburn University</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial and Systems Engineering</t>
+          <t>Department of Mechanical Engineering</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: while housed in Industrial and Systems Engineering with a broad mention of transportation applications, the primary departmental focus and hiring emphasis is strictly on Industrialized Construction.</t>
+          <t>Low fit: position is in Mechanical Engineering and lacks description details, which does not align with the candidate's transportation engineering and planning profile.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+          <t>Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -3016,12 +3016,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Gainesville, FL</t>
+          <t>Auburn, AL</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3031,17 +3031,17 @@
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>The Department of Industrial and Systems Engineering at the University of Florida seeks a tenured/tenure-track faculty member specializing in Industrialized Construction with a PhD in ISE, Manufacturing Engineering, Civil Engineering, Mechanical Engineering, or a closely related field. | Research Topics: Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+          <t>An open-rank faculty position in mechanical engineering requiring a Ph.D. in mechanical engineering or a closely related field. | Research Topics: Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-industrial-systems-engineering-at-university-of-florida-4323668785</t>
+          <t>https://engineering.academickeys.com/job/f320isty/AssistantAssociateFull-Professor</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P28" s="3" t="inlineStr">
@@ -3060,44 +3060,44 @@
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>29.6436</v>
+        <v>32.5919529</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>-82.3549</v>
+        <v>-85.4959775</v>
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>56d501f448e77e05</t>
+          <t>c08698a4bf95171b</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Supply Chain Management</t>
+          <t>Assistant / Associate Professor of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>University of Washington</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>J.B. Hunt Transport Department of Supply Chain Management, Sam M. Walton College of Business</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>3</v>
+          <t>Industrial and Systems Engineering</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>7</v>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Low fit: Business school faculty position focused entirely on defense-relevant supply chain management and contested logistics, which falls outside transportation engineering.</t>
+          <t>Strong interdisciplinary match: industrial and systems engineering position in a target department, though specific mobility focus depends on the full department scope.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
+          <t>Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -3107,12 +3107,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -3122,17 +3122,17 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>The Sam M. Walton College of Business at the University of Arkansas seeks two tenure-track Assistant Professors in Supply Chain Management as part of a faculty cluster hire focused on contested logistics and defense-relevant supply chains. | Research Topics: Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
+          <t>Assistant or Associate Professor position in Industrial and Systems Engineering requiring a Ph.D. in a relevant engineering or analytical discipline. | Research Topics: Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-two-open-positions-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460109211</t>
+          <t>https://engineering.academickeys.com/job/g4m97a60/AssistantAssociate-Professor-Industrial-and-Systems-Engineering-Systems-Engineering-Focus</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -3151,54 +3151,54 @@
         </is>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>36.0625843</v>
+        <v>47.6553</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>-94.1574328</v>
+        <v>-122.3035</v>
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>8b974c86c7dfa1c1</t>
+          <t>9d5682cf4dbca334</t>
         </is>
       </c>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Supply Chain Management</t>
+          <t>Professor &amp; Department Chair</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Iowa State University</t>
+          <t>University of Pittsburgh</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Department of Supply Chain Management, Ivy College of Business</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>6</v>
+          <t>Department of Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: the role is in a business school supply chain department rather than engineering or planning, though it accepts transportation as a related specialization.</t>
+          <t>Low fit: departmental leadership position for a broad Civil and Environmental Engineering department rather than a dedicated transportation research faculty role.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Transportation, Logistics, Operations</t>
+          <t>Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Tenured</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Ames, IA</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -3213,17 +3213,17 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>The Ivy College of Business at Iowa State University seeks a tenure-track Assistant Professor in Supply Chain Management to conduct research and teach across undergraduate, master's, and Ph.D. levels, requiring a Ph.D. in business administration or a related field such as transportation or logistics. | Research Topics: Supply Chain Management, Transportation, Logistics, Operations</t>
+          <t>Strictly 1 concise sentence summarizing the primary focus of the role and minimum degree qualification. | Research Topics: Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-in-supply-chain-management-at-iowa-state-university-ivy-college-of-business-4440811209</t>
+          <t>http://engineering.academickeys.com/job/vhlo0w6p/Professor--Department-Chair--Electrical-and-Computer-Engineering</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P30" s="3" t="inlineStr">
@@ -3242,79 +3242,79 @@
         </is>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>42.0267567</v>
+        <v>40.444153</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>-93.6170448</v>
+        <v>-79.962461</v>
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>e994e392d38b77ce</t>
+          <t>17acd4b4e7207871</t>
         </is>
       </c>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Operations Management</t>
+          <t>Lecturer in Discipline or Senior Lecturer in Discipline</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>University of Illinois Chicago</t>
+          <t>Columbia University</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Department of Information and Decision Sciences, College of Business Administration</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>7</v>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match in a Business School department that explicitly prioritizes transportation and AI in supply chain management as a preferred research domain.</t>
+          <t>Moderate fit: general lecturer position at Columbia University in an unspecified discipline, requiring further text details to confirm a transportation focus.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
+          <t>Higher Education, Instruction, Academic Teaching</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>2026-12-06</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>$185,000 - $220,000 annually</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>The Department of Information and Decision Sciences seeks a tenure-track Assistant Professor in Operations Management with a preferred research focus on transportation and AI-driven supply chain management, requiring a Ph.D. in Management Science, Operations Management, Operations Research, or a closely related field. | Research Topics: Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
+          <t>This is a faculty teaching role at Columbia University, though the specific academic department and subject focus are missing from the current snippet. | Research Topics: Higher Education, Instruction, Academic Teaching</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-ids-supply-chain-operations-management-at-university-of-illinois-chicago-4463632919</t>
+          <t>http://engineering.academickeys.com/job/arsy3jqh/Open-Rank-Lecturer-in-Discipline-or-Senior-Lecturer-in-Discipline</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P31" s="3" t="inlineStr">
@@ -3333,44 +3333,44 @@
         </is>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>41.8748613</v>
+        <v>40.8077507</v>
       </c>
       <c r="R31" s="2" t="n">
-        <v>-87.6519866</v>
+        <v>-73.9624901</v>
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>d58da246ce5b68ab</t>
+          <t>f11b4a4e74422ae3</t>
         </is>
       </c>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Public Policy (Market-Based Solutions to Societal Challenges)</t>
+          <t>Assistant/Associate Professor of Civil Engineering</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Madison</t>
+          <t>Cedarville University</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>La Follette School of Public Affairs, College of Letters &amp; Science</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>3</v>
+          <t>Department of Civil Engineering</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Low fit: Public policy and economics faculty position focused on market-based solutions, though transportation and infrastructure finance is listed as one of many broad application areas.</t>
+          <t>Moderate fit: broad Civil Engineering search where transportation may be acceptable, but lacks a dedicated job description snippet for precise evaluation.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
+          <t>Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -3380,12 +3380,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Madison, WI</t>
+          <t>Cedarville, OH</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -3395,17 +3395,17 @@
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>The La Follette School of Public Affairs at UW-Madison seeks a tenure-track assistant professor to conduct theoretically grounded research on market-based solutions and incentive-compatible policy design across various domains. | Research Topics: Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
+          <t>A faculty position in civil engineering requiring a Ph.D. to teach undergraduate courses and engage in scholarly activity. | Research Topics: Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-public-policy-market-based-solutions-to-societal-challenges-at-uw-madison-college-of-letters-science-4435310692</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179544290&amp;Title=Assistant%2FAssociate%20Professor%20of%20Civil%20Engineering</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>HigherEdJobs</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -3424,54 +3424,54 @@
         </is>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>43.07469</v>
+        <v>39.7540491</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>-89.3841663</v>
+        <v>-83.8170518</v>
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>886b76b05d362fdc</t>
+          <t>751c7406865a2787</t>
         </is>
       </c>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Multiple Faculty Positions in Computer Science and Engineering</t>
+          <t>Assistant Professor of Information and Decision Sciences (Supply Chain &amp; Operations Management)</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Texas A&amp;M University</t>
+          <t>University of Illinois Chicago</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Department of Computer Science and Engineering</t>
+          <t>Information and Decision Sciences (IDS)</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: open faculty search in Computer Science and Engineering without explicit specialization in transportation or mobility systems.</t>
+          <t>Low fit: position is in Supply Chain and Operations Management within a business school, which falls outside the candidate's core transportation engineering and mobility systems profile.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
+          <t>Supply Chain Management, Operations Management, Decision Sciences</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>College Station, TX</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -3486,22 +3486,22 @@
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Texas A&amp;M University invites applications for multiple faculty positions in Computer Science and Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
+          <t>This is a tenure-track Assistant Professor role in Supply Chain and Operations Management requiring a Ph.D. in a relevant business or analytical discipline. | Research Topics: Supply Chain Management, Operations Management, Decision Sciences</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>http://engineering.academickeys.com/job/rh7lvag4/CSE--TAMU-Multiple-Faculty-Positions</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179552436&amp;Title=Assistant%20Professor%20%2D%20IDS%20%28Supply%20Chain%20%26%20Operations%20Management%29</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>AcademicKeys</t>
+          <t>HigherEdJobs</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -3515,54 +3515,54 @@
         </is>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>30.6187</v>
+        <v>41.8748613</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>-96.3365</v>
+        <v>-87.6519866</v>
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>7d5d844d65485b4b</t>
+          <t>77e0632bd4e74eae</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Civil Engineering</t>
+          <t>Professor, Associate Professor, or Assistant Professor of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>McNeese State University</t>
+          <t>Auburn University</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="n">
-        <v>5</v>
+          <t>Department of Industrial and Systems Engineering</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: broad Civil Engineering search where transportation is not explicitly prioritized in the snippet.</t>
+          <t>Moderate fit: Industrial and Systems Engineering faculty position at Auburn University, but the job description text was missing to confirm a specific focus on mobility systems.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Engineering Education</t>
+          <t>Industrial Engineering, Systems Engineering, Operations Research</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Lake Charles, LA</t>
+          <t>Auburn, AL</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -3572,17 +3572,17 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>$76,000 per year</t>
+          <t>$80,000 - $180,000 per year</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Assistant Professor position in Civil and Environmental Engineering at McNeese State University with a salary of $76,000 per year. | Research Topics: Civil Engineering, Engineering Education</t>
+          <t>Open-rank faculty position in Industrial and Systems Engineering requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Systems Engineering, Operations Research</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545361&amp;Title=Assistant%20Professor%20of%20Civil%20Engineering</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179548357&amp;Title=Professor%2C%20Associate%20Professor%2C%20Assistant%20Professor%20%2D%20Industrial%20and%20Systems%20Engineering</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -3606,105 +3606,1197 @@
         </is>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>30.1751363</v>
+        <v>32.5919529</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>-93.2112786</v>
+        <v>-85.4959775</v>
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>bd292fb9f52ac2e9</t>
+          <t>d0f23a527bf71c22</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>Teaching Assistant Professor</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>University of Arkansas</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit: Broad Civil Engineering faculty search where transportation is only one of multiple acceptable sub-disciplines.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Civil Engineering Education, Transportation Engineering</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Non-Tenure Track</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Fayetteville, AR</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>A teaching-focused assistant professor position in civil engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Civil Engineering Education, Transportation Engineering</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179541925&amp;Title=Teaching%20Assistant%20Professor</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>HigherEdJobs</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P35" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>36.0970389</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>-94.1703322</v>
+      </c>
+      <c r="S35" s="2" t="inlineStr">
+        <is>
+          <t>8b28f5b58e7e3607</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Teaching</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Florida Atlantic University</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Department of Civil, Environmental &amp; Geomatics Engineering</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit: it is a Civil Engineering teaching position in a department with transportation research centers, but requires teaching structural analysis and design-related classes alongside a P.E. license.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Non-Tenure Track</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Boca Raton, FL</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Commensurate with Experience</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>This is a non-tenure-track Assistant Teaching Professor position in civil engineering requiring a Ph.D. and P.E. license to teach undergraduate and graduate courses including structural analysis and design. | Research Topics: Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-teaching-at-florida-atlantic-university-4414964381</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="n">
+        <v>26.1194058</v>
+      </c>
+      <c r="R36" s="2" t="n">
+        <v>-80.14167999999999</v>
+      </c>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>7bdaa996cf64d1f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Assistant or Associate Professor in Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>University of Arkansas</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>J.B. Hunt Transport Department of Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Low fit: this is a faculty position in Supply Chain Management within a Business School rather than Transportation Engineering.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Supply Chain Management, Logistics, Operations Research</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Fayetteville, AR</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>This is a tenure-track Assistant or Associate Professor position in Supply Chain Management requiring a strong research record in leading peer-reviewed journals. | Research Topics: Supply Chain Management, Logistics, Operations Research</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-or-associate-professor-open-rank-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460111187</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>36.0625843</v>
+      </c>
+      <c r="R37" s="2" t="n">
+        <v>-94.1574328</v>
+      </c>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>c16a694d5f7f68d4</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Aerospace Engineering</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>The University of Kansas</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Department of Aerospace Engineering</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>The position is specifically for Aerospace Engineering focusing on aircraft and space systems, where the candidate's core transportation engineering expertise is not the primary requirement.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Lawrence, KS</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>This is a tenure-track faculty position in Aerospace Engineering requiring a doctorate in Aerospace Engineering or a closely related field, focusing on aviation and space-related research. | Research Topics: Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-aerospace-engineering-at-the-university-of-kansas-4460398978</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>39.0559267</v>
+      </c>
+      <c r="R38" s="2" t="n">
+        <v>-94.6090332</v>
+      </c>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>4a53cfad86712a72</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Assistant/Associate/Full Professor in Industrial and Systems Engineering</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>University of Florida</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Department of Industrial and Systems Engineering</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit: while housed in Industrial and Systems Engineering with a broad mention of transportation applications, the primary departmental focus and hiring emphasis is strictly on Industrialized Construction.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Gainesville, FL</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>The Department of Industrial and Systems Engineering at the University of Florida seeks a tenured/tenure-track faculty member specializing in Industrialized Construction with a PhD in ISE, Manufacturing Engineering, Civil Engineering, Mechanical Engineering, or a closely related field. | Research Topics: Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-industrial-systems-engineering-at-university-of-florida-4323668785</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="P39" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>29.6436</v>
+      </c>
+      <c r="R39" s="2" t="n">
+        <v>-82.3549</v>
+      </c>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>56d501f448e77e05</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="26" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor in Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>University of Arkansas</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>J.B. Hunt Transport Department of Supply Chain Management, Sam M. Walton College of Business</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Low fit: Business school faculty position focused entirely on defense-relevant supply chain management and contested logistics, which falls outside transportation engineering.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Fayetteville, AR</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>The Sam M. Walton College of Business at the University of Arkansas seeks two tenure-track Assistant Professors in Supply Chain Management as part of a faculty cluster hire focused on contested logistics and defense-relevant supply chains. | Research Topics: Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-two-open-positions-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460109211</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="n">
+        <v>36.0625843</v>
+      </c>
+      <c r="R40" s="2" t="n">
+        <v>-94.1574328</v>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>8b974c86c7dfa1c1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor in Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Iowa State University</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Department of Supply Chain Management, Ivy College of Business</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit: the role is in a business school supply chain department rather than engineering or planning, though it accepts transportation as a related specialization.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Supply Chain Management, Transportation, Logistics, Operations</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Ames, IA</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>The Ivy College of Business at Iowa State University seeks a tenure-track Assistant Professor in Supply Chain Management to conduct research and teach across undergraduate, master's, and Ph.D. levels, requiring a Ph.D. in business administration or a related field such as transportation or logistics. | Research Topics: Supply Chain Management, Transportation, Logistics, Operations</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-in-supply-chain-management-at-iowa-state-university-ivy-college-of-business-4440811209</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>42.0267567</v>
+      </c>
+      <c r="R41" s="2" t="n">
+        <v>-93.6170448</v>
+      </c>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>e994e392d38b77ce</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor in Operations Management</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>University of Illinois Chicago</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Department of Information and Decision Sciences, College of Business Administration</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Strong interdisciplinary match in a Business School department that explicitly prioritizes transportation and AI in supply chain management as a preferred research domain.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>2026-12-06</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>$185,000 - $220,000 annually</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>The Department of Information and Decision Sciences seeks a tenure-track Assistant Professor in Operations Management with a preferred research focus on transportation and AI-driven supply chain management, requiring a Ph.D. in Management Science, Operations Management, Operations Research, or a closely related field. | Research Topics: Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-ids-supply-chain-operations-management-at-university-of-illinois-chicago-4463632919</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="P42" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>41.8748613</v>
+      </c>
+      <c r="R42" s="2" t="n">
+        <v>-87.6519866</v>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>d58da246ce5b68ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Public Policy (Market-Based Solutions to Societal Challenges)</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>University of Wisconsin-Madison</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>La Follette School of Public Affairs, College of Letters &amp; Science</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Low fit: Public policy and economics faculty position focused on market-based solutions, though transportation and infrastructure finance is listed as one of many broad application areas.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Madison, WI</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>The La Follette School of Public Affairs at UW-Madison seeks a tenure-track assistant professor to conduct theoretically grounded research on market-based solutions and incentive-compatible policy design across various domains. | Research Topics: Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-public-policy-market-based-solutions-to-societal-challenges-at-uw-madison-college-of-letters-science-4435310692</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>43.07469</v>
+      </c>
+      <c r="R43" s="2" t="n">
+        <v>-89.3841663</v>
+      </c>
+      <c r="S43" s="2" t="inlineStr">
+        <is>
+          <t>886b76b05d362fdc</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Multiple Faculty Positions in Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Texas A&amp;M University</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Department of Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit: open faculty search in Computer Science and Engineering without explicit specialization in transportation or mobility systems.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>College Station, TX</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>Texas A&amp;M University invites applications for multiple faculty positions in Computer Science and Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>http://engineering.academickeys.com/job/rh7lvag4/CSE--TAMU-Multiple-Faculty-Positions</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>AcademicKeys</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>30.6187</v>
+      </c>
+      <c r="R44" s="2" t="n">
+        <v>-96.3365</v>
+      </c>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>7d5d844d65485b4b</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Civil Engineering</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>McNeese State University</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit: broad Civil Engineering search where transportation is not explicitly prioritized in the snippet.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Civil Engineering, Engineering Education</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Lake Charles, LA</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>$76,000 per year</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>Assistant Professor position in Civil and Environmental Engineering at McNeese State University with a salary of $76,000 per year. | Research Topics: Civil Engineering, Engineering Education</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545361&amp;Title=Assistant%20Professor%20of%20Civil%20Engineering</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>HigherEdJobs</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P45" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>30.1751363</v>
+      </c>
+      <c r="R45" s="2" t="n">
+        <v>-93.2112786</v>
+      </c>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>bd292fb9f52ac2e9</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>Tenure-Track Faculty Positions in Transportation Engineering</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>National Taiwan University</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Department of Civil Engineering</t>
         </is>
       </c>
-      <c r="D35" s="7" t="n">
+      <c r="D46" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>Core match: seeks multiple tenure-track faculty positions specifically in the Transportation track within a Department of Civil Engineering.</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Transportation Engineering, Mobility Systems, Transit Planning</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G46" s="3" t="inlineStr">
         <is>
           <t>Tenure-Track</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Taipei, Taiwan</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="I46" s="3" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>NT$83,720–137,370 monthly</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="K46" s="4" t="inlineStr">
         <is>
           <t>The Department of Civil Engineering at National Taiwan University invites applications for multiple tenure-track faculty positions in Transportation Engineering. | Research Topics: Transportation Engineering, Mobility Systems, Transit Planning</t>
         </is>
       </c>
-      <c r="L35" s="5" t="inlineStr">
+      <c r="L46" s="5" t="inlineStr">
         <is>
           <t>https://jobs.chronicle.com/job/38034402/faculty-recruitment-announcement-department-of-civil-engineering-national-taiwan-university/</t>
         </is>
       </c>
-      <c r="M35" s="3" t="inlineStr">
+      <c r="M46" s="3" t="inlineStr">
         <is>
           <t>Chronicle</t>
         </is>
       </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O35" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P35" s="3" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="Q35" s="2" t="n">
+      <c r="Q46" s="2" t="n">
         <v>25.0375198</v>
       </c>
-      <c r="R35" s="2" t="n">
+      <c r="R46" s="2" t="n">
         <v>121.5636796</v>
       </c>
-      <c r="S35" s="2" t="inlineStr">
+      <c r="S46" s="2" t="inlineStr">
         <is>
           <t>f056997ace2e1de7</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Public Policy and Administration</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>University of Texas at Arlington</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Department of Public Affairs &amp; Planning</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit: Assistant Professor in Public Affairs &amp; Planning focused on public policy and urban studies, offering potential interdisciplinary overlap despite lacking a specific transportation mandate.</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Arlington, TX</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>The University of Texas at Arlington seeks a tenure-track Assistant Professor in Public Policy &amp; Planning to conduct policy research, secure external funding, and teach public administration courses requiring a Ph.D. | Research Topics: Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-at-excel-campus-activities-4464851831</t>
+        </is>
+      </c>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="P47" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>32.7315155</v>
+      </c>
+      <c r="R47" s="2" t="n">
+        <v>-97.1171533</v>
+      </c>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>15704bb25858281c</t>
         </is>
       </c>
     </row>
@@ -3744,6 +4836,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert map to MarkerCluster job count aggregation and enhance cross-board deduplication for Wisconsin and UIC
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -493,12 +493,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="95" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
     <col width="151" customWidth="1" min="6" max="6"/>
@@ -3438,30 +3438,30 @@
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Information and Decision Sciences (Supply Chain &amp; Operations Management)</t>
+          <t>Professor, Associate Professor, or Assistant Professor of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>University of Illinois Chicago</t>
+          <t>Auburn University</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Information and Decision Sciences (IDS)</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>3</v>
+          <t>Department of Industrial and Systems Engineering</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Low fit: position is in Supply Chain and Operations Management within a business school, which falls outside the candidate's core transportation engineering and mobility systems profile.</t>
+          <t>Moderate fit: Industrial and Systems Engineering faculty position at Auburn University, but the job description text was missing to confirm a specific focus on mobility systems.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Operations Management, Decision Sciences</t>
+          <t>Industrial Engineering, Systems Engineering, Operations Research</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Auburn, AL</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$80,000 - $180,000 per year</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track Assistant Professor role in Supply Chain and Operations Management requiring a Ph.D. in a relevant business or analytical discipline. | Research Topics: Supply Chain Management, Operations Management, Decision Sciences</t>
+          <t>Open-rank faculty position in Industrial and Systems Engineering requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Systems Engineering, Operations Research</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179552436&amp;Title=Assistant%20Professor%20%2D%20IDS%20%28Supply%20Chain%20%26%20Operations%20Management%29</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179548357&amp;Title=Professor%2C%20Associate%20Professor%2C%20Assistant%20Professor%20%2D%20Industrial%20and%20Systems%20Engineering</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -3515,54 +3515,54 @@
         </is>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>41.8748613</v>
+        <v>32.5919529</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>-87.6519866</v>
+        <v>-85.4959775</v>
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>77e0632bd4e74eae</t>
+          <t>d0f23a527bf71c22</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Professor, Associate Professor, or Assistant Professor of Industrial and Systems Engineering</t>
+          <t>Teaching Assistant Professor</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Auburn University</t>
+          <t>University of Arkansas</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial and Systems Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="D34" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: Industrial and Systems Engineering faculty position at Auburn University, but the job description text was missing to confirm a specific focus on mobility systems.</t>
+          <t>Moderate fit: Broad Civil Engineering faculty search where transportation is only one of multiple acceptable sub-disciplines.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Industrial Engineering, Systems Engineering, Operations Research</t>
+          <t>Civil Engineering Education, Transportation Engineering</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Auburn, AL</t>
+          <t>Fayetteville, AR</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -3572,17 +3572,17 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>$80,000 - $180,000 per year</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Open-rank faculty position in Industrial and Systems Engineering requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Systems Engineering, Operations Research</t>
+          <t>A teaching-focused assistant professor position in civil engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Civil Engineering Education, Transportation Engineering</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179548357&amp;Title=Professor%2C%20Associate%20Professor%2C%20Assistant%20Professor%20%2D%20Industrial%20and%20Systems%20Engineering</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179541925&amp;Title=Teaching%20Assistant%20Professor</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
@@ -3606,31 +3606,31 @@
         </is>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>32.5919529</v>
+        <v>36.0970389</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>-85.4959775</v>
+        <v>-94.1703322</v>
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>d0f23a527bf71c22</t>
+          <t>8b28f5b58e7e3607</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Teaching Assistant Professor</t>
+          <t>Assistant Professor of Teaching</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>Florida Atlantic University</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Department of Civil, Environmental &amp; Geomatics Engineering</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
@@ -3638,12 +3638,12 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: Broad Civil Engineering faculty search where transportation is only one of multiple acceptable sub-disciplines.</t>
+          <t>Moderate fit: it is a Civil Engineering teaching position in a department with transportation research centers, but requires teaching structural analysis and design-related classes alongside a P.E. license.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering Education, Transportation Engineering</t>
+          <t>Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
+          <t>Boca Raton, FL</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -3663,22 +3663,22 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Commensurate with Experience</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>A teaching-focused assistant professor position in civil engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Civil Engineering Education, Transportation Engineering</t>
+          <t>This is a non-tenure-track Assistant Teaching Professor position in civil engineering requiring a Ph.D. and P.E. license to teach undergraduate and graduate courses including structural analysis and design. | Research Topics: Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179541925&amp;Title=Teaching%20Assistant%20Professor</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-teaching-at-florida-atlantic-university-4414964381</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>HigherEdJobs</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="P35" s="3" t="inlineStr">
@@ -3697,74 +3697,74 @@
         </is>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>36.0970389</v>
+        <v>26.1194058</v>
       </c>
       <c r="R35" s="2" t="n">
-        <v>-94.1703322</v>
+        <v>-80.14167999999999</v>
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>8b28f5b58e7e3607</t>
+          <t>7bdaa996cf64d1f6</t>
         </is>
       </c>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Teaching</t>
+          <t>Assistant or Associate Professor in Supply Chain Management</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Florida Atlantic University</t>
+          <t>University of Arkansas</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil, Environmental &amp; Geomatics Engineering</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="n">
-        <v>5</v>
+          <t>J.B. Hunt Transport Department of Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: it is a Civil Engineering teaching position in a department with transportation research centers, but requires teaching structural analysis and design-related classes alongside a P.E. license.</t>
+          <t>Low fit: this is a faculty position in Supply Chain Management within a Business School rather than Transportation Engineering.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+          <t>Supply Chain Management, Logistics, Operations Research</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Non-Tenure Track</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Boca Raton, FL</t>
+          <t>Fayetteville, AR</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Commensurate with Experience</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>This is a non-tenure-track Assistant Teaching Professor position in civil engineering requiring a Ph.D. and P.E. license to teach undergraduate and graduate courses including structural analysis and design. | Research Topics: Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+          <t>This is a tenure-track Assistant or Associate Professor position in Supply Chain Management requiring a strong research record in leading peer-reviewed journals. | Research Topics: Supply Chain Management, Logistics, Operations Research</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-teaching-at-florida-atlantic-university-4414964381</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-or-associate-professor-open-rank-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460111187</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P36" s="3" t="inlineStr">
@@ -3788,31 +3788,31 @@
         </is>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>26.1194058</v>
+        <v>36.0625843</v>
       </c>
       <c r="R36" s="2" t="n">
-        <v>-80.14167999999999</v>
+        <v>-94.1574328</v>
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>7bdaa996cf64d1f6</t>
+          <t>c16a694d5f7f68d4</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Assistant or Associate Professor in Supply Chain Management</t>
+          <t>Assistant Professor of Aerospace Engineering</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>The University of Kansas</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>J.B. Hunt Transport Department of Supply Chain Management</t>
+          <t>Department of Aerospace Engineering</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -3820,12 +3820,12 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Low fit: this is a faculty position in Supply Chain Management within a Business School rather than Transportation Engineering.</t>
+          <t>The position is specifically for Aerospace Engineering focusing on aircraft and space systems, where the candidate's core transportation engineering expertise is not the primary requirement.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Logistics, Operations Research</t>
+          <t>Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -3835,12 +3835,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
+          <t>Lawrence, KS</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3850,12 +3850,12 @@
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track Assistant or Associate Professor position in Supply Chain Management requiring a strong research record in leading peer-reviewed journals. | Research Topics: Supply Chain Management, Logistics, Operations Research</t>
+          <t>This is a tenure-track faculty position in Aerospace Engineering requiring a doctorate in Aerospace Engineering or a closely related field, focusing on aviation and space-related research. | Research Topics: Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-or-associate-professor-open-rank-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460111187</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-aerospace-engineering-at-the-university-of-kansas-4460398978</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr">
@@ -3879,44 +3879,44 @@
         </is>
       </c>
       <c r="Q37" s="2" t="n">
-        <v>36.0625843</v>
+        <v>39.0559267</v>
       </c>
       <c r="R37" s="2" t="n">
-        <v>-94.1574328</v>
+        <v>-94.6090332</v>
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>c16a694d5f7f68d4</t>
+          <t>4a53cfad86712a72</t>
         </is>
       </c>
     </row>
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Aerospace Engineering</t>
+          <t>Assistant/Associate/Full Professor in Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>The University of Kansas</t>
+          <t>University of Florida</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Department of Aerospace Engineering</t>
+          <t>Department of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>The position is specifically for Aerospace Engineering focusing on aircraft and space systems, where the candidate's core transportation engineering expertise is not the primary requirement.</t>
+          <t>Moderate fit: while housed in Industrial and Systems Engineering with a broad mention of transportation applications, the primary departmental focus and hiring emphasis is strictly on Industrialized Construction.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+          <t>Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -3926,27 +3926,27 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Lawrence, KS</t>
+          <t>Gainesville, FL</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track faculty position in Aerospace Engineering requiring a doctorate in Aerospace Engineering or a closely related field, focusing on aviation and space-related research. | Research Topics: Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+          <t>The Department of Industrial and Systems Engineering at the University of Florida seeks a tenured/tenure-track faculty member specializing in Industrialized Construction with a PhD in ISE, Manufacturing Engineering, Civil Engineering, Mechanical Engineering, or a closely related field. | Research Topics: Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-aerospace-engineering-at-the-university-of-kansas-4460398978</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-industrial-systems-engineering-at-university-of-florida-4323668785</t>
         </is>
       </c>
       <c r="M38" s="3" t="inlineStr">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="P38" s="3" t="inlineStr">
@@ -3970,44 +3970,44 @@
         </is>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>39.0559267</v>
+        <v>29.6436</v>
       </c>
       <c r="R38" s="2" t="n">
-        <v>-94.6090332</v>
+        <v>-82.3549</v>
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>4a53cfad86712a72</t>
+          <t>56d501f448e77e05</t>
         </is>
       </c>
     </row>
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate/Full Professor in Industrial and Systems Engineering</t>
+          <t>Assistant Professor in Supply Chain Management</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>University of Florida</t>
+          <t>Iowa State University</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial and Systems Engineering</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>4</v>
+          <t>Department of Supply Chain Management, Ivy College of Business</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: while housed in Industrial and Systems Engineering with a broad mention of transportation applications, the primary departmental focus and hiring emphasis is strictly on Industrialized Construction.</t>
+          <t>Moderate fit: the role is in a business school supply chain department rather than engineering or planning, though it accepts transportation as a related specialization.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+          <t>Supply Chain Management, Transportation, Logistics, Operations</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Gainesville, FL</t>
+          <t>Ames, IA</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -4032,12 +4032,12 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>The Department of Industrial and Systems Engineering at the University of Florida seeks a tenured/tenure-track faculty member specializing in Industrialized Construction with a PhD in ISE, Manufacturing Engineering, Civil Engineering, Mechanical Engineering, or a closely related field. | Research Topics: Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+          <t>The Ivy College of Business at Iowa State University seeks a tenure-track Assistant Professor in Supply Chain Management to conduct research and teach across undergraduate, master's, and Ph.D. levels, requiring a Ph.D. in business administration or a related field such as transportation or logistics. | Research Topics: Supply Chain Management, Transportation, Logistics, Operations</t>
         </is>
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-industrial-systems-engineering-at-university-of-florida-4323668785</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-in-supply-chain-management-at-iowa-state-university-ivy-college-of-business-4440811209</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr">
@@ -4061,59 +4061,59 @@
         </is>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>29.6436</v>
+        <v>42.0267567</v>
       </c>
       <c r="R39" s="2" t="n">
-        <v>-82.3549</v>
+        <v>-93.6170448</v>
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>56d501f448e77e05</t>
+          <t>e994e392d38b77ce</t>
         </is>
       </c>
     </row>
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Supply Chain Management</t>
+          <t>Multiple Faculty Positions in Computer Science and Engineering</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>Texas A&amp;M University</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>J.B. Hunt Transport Department of Supply Chain Management, Sam M. Walton College of Business</t>
+          <t>Department of Computer Science and Engineering</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Low fit: Business school faculty position focused entirely on defense-relevant supply chain management and contested logistics, which falls outside transportation engineering.</t>
+          <t>Moderate fit: open faculty search in Computer Science and Engineering without explicit specialization in transportation or mobility systems.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
+          <t>Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
+          <t>College Station, TX</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -4123,22 +4123,22 @@
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>The Sam M. Walton College of Business at the University of Arkansas seeks two tenure-track Assistant Professors in Supply Chain Management as part of a faculty cluster hire focused on contested logistics and defense-relevant supply chains. | Research Topics: Supply Chain Management, Contested Logistics, Military and Defense Logistics, National Security Supply Chains</t>
+          <t>Texas A&amp;M University invites applications for multiple faculty positions in Computer Science and Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-two-open-positions-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460109211</t>
+          <t>http://engineering.academickeys.com/job/rh7lvag4/CSE--TAMU-Multiple-Faculty-Positions</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
@@ -4152,54 +4152,54 @@
         </is>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>36.0625843</v>
+        <v>30.6187</v>
       </c>
       <c r="R40" s="2" t="n">
-        <v>-94.1574328</v>
+        <v>-96.3365</v>
       </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
-          <t>8b974c86c7dfa1c1</t>
+          <t>7d5d844d65485b4b</t>
         </is>
       </c>
     </row>
     <row r="41" ht="26" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Supply Chain Management</t>
+          <t>Assistant Professor of Civil Engineering</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Iowa State University</t>
+          <t>McNeese State University</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Department of Supply Chain Management, Ivy College of Business</t>
+          <t>Civil and Environmental Engineering</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: the role is in a business school supply chain department rather than engineering or planning, though it accepts transportation as a related specialization.</t>
+          <t>Moderate fit: broad Civil Engineering search where transportation is not explicitly prioritized in the snippet.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Transportation, Logistics, Operations</t>
+          <t>Civil Engineering, Engineering Education</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Ames, IA</t>
+          <t>Lake Charles, LA</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -4209,32 +4209,32 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$76,000 per year</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>The Ivy College of Business at Iowa State University seeks a tenure-track Assistant Professor in Supply Chain Management to conduct research and teach across undergraduate, master's, and Ph.D. levels, requiring a Ph.D. in business administration or a related field such as transportation or logistics. | Research Topics: Supply Chain Management, Transportation, Logistics, Operations</t>
+          <t>Assistant Professor position in Civil and Environmental Engineering at McNeese State University with a salary of $76,000 per year. | Research Topics: Civil Engineering, Engineering Education</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-in-supply-chain-management-at-iowa-state-university-ivy-college-of-business-4440811209</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545361&amp;Title=Assistant%20Professor%20of%20Civil%20Engineering</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>HigherEdJobs</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P41" s="3" t="inlineStr">
@@ -4243,44 +4243,44 @@
         </is>
       </c>
       <c r="Q41" s="2" t="n">
-        <v>42.0267567</v>
+        <v>30.1751363</v>
       </c>
       <c r="R41" s="2" t="n">
-        <v>-93.6170448</v>
+        <v>-93.2112786</v>
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>e994e392d38b77ce</t>
+          <t>bd292fb9f52ac2e9</t>
         </is>
       </c>
     </row>
     <row r="42" ht="26" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Operations Management</t>
+          <t>Tenure-Track Faculty Positions in Transportation Engineering</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>University of Illinois Chicago</t>
+          <t>National Taiwan University</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Department of Information and Decision Sciences, College of Business Administration</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="n">
-        <v>7</v>
+          <t>Department of Civil Engineering</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>9</v>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match in a Business School department that explicitly prioritizes transportation and AI in supply chain management as a preferred research domain.</t>
+          <t>Core match: seeks multiple tenure-track faculty positions specifically in the Transportation track within a Department of Civil Engineering.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
+          <t>Transportation Engineering, Mobility Systems, Transit Planning</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -4290,42 +4290,42 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Taipei, Taiwan</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>2026-12-06</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>$185,000 - $220,000 annually</t>
+          <t>NT$83,720–137,370 monthly</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>The Department of Information and Decision Sciences seeks a tenure-track Assistant Professor in Operations Management with a preferred research focus on transportation and AI-driven supply chain management, requiring a Ph.D. in Management Science, Operations Management, Operations Research, or a closely related field. | Research Topics: Operations Management, Transportation, Supply Chain Management, Artificial Intelligence and Analytics</t>
+          <t>The Department of Civil Engineering at National Taiwan University invites applications for multiple tenure-track faculty positions in Transportation Engineering. | Research Topics: Transportation Engineering, Mobility Systems, Transit Planning</t>
         </is>
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-%E2%80%93-ids-supply-chain-operations-management-at-university-of-illinois-chicago-4463632919</t>
+          <t>https://jobs.chronicle.com/job/38034402/faculty-recruitment-announcement-department-of-civil-engineering-national-taiwan-university/</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P42" s="3" t="inlineStr">
@@ -4334,44 +4334,44 @@
         </is>
       </c>
       <c r="Q42" s="2" t="n">
-        <v>41.8748613</v>
+        <v>25.0375198</v>
       </c>
       <c r="R42" s="2" t="n">
-        <v>-87.6519866</v>
+        <v>121.5636796</v>
       </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
-          <t>d58da246ce5b68ab</t>
+          <t>f056997ace2e1de7</t>
         </is>
       </c>
     </row>
     <row r="43" ht="26" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Public Policy (Market-Based Solutions to Societal Challenges)</t>
+          <t>Assistant Professor of Public Policy and Administration</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Madison</t>
+          <t>University of Texas at Arlington</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>La Follette School of Public Affairs, College of Letters &amp; Science</t>
+          <t>Department of Public Affairs &amp; Planning</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Low fit: Public policy and economics faculty position focused on market-based solutions, though transportation and infrastructure finance is listed as one of many broad application areas.</t>
+          <t>Moderate fit: Assistant Professor in Public Affairs &amp; Planning focused on public policy and urban studies, offering potential interdisciplinary overlap despite lacking a specific transportation mandate.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
+          <t>Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Madison, WI</t>
+          <t>Arlington, TX</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -4396,12 +4396,12 @@
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>The La Follette School of Public Affairs at UW-Madison seeks a tenure-track assistant professor to conduct theoretically grounded research on market-based solutions and incentive-compatible policy design across various domains. | Research Topics: Market-based institutions, Public policy analysis, Transportation and infrastructure finance, Institutional design</t>
+          <t>The University of Texas at Arlington seeks a tenure-track Assistant Professor in Public Policy &amp; Planning to conduct policy research, secure external funding, and teach public administration courses requiring a Ph.D. | Research Topics: Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
         </is>
       </c>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-public-policy-market-based-solutions-to-societal-challenges-at-uw-madison-college-of-letters-science-4435310692</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-at-excel-campus-activities-4464851831</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
@@ -4425,376 +4425,12 @@
         </is>
       </c>
       <c r="Q43" s="2" t="n">
-        <v>43.07469</v>
+        <v>32.7315155</v>
       </c>
       <c r="R43" s="2" t="n">
-        <v>-89.3841663</v>
+        <v>-97.1171533</v>
       </c>
       <c r="S43" s="2" t="inlineStr">
-        <is>
-          <t>886b76b05d362fdc</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Multiple Faculty Positions in Computer Science and Engineering</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Texas A&amp;M University</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Department of Computer Science and Engineering</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>Moderate fit: open faculty search in Computer Science and Engineering without explicit specialization in transportation or mobility systems.</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>College Station, TX</t>
-        </is>
-      </c>
-      <c r="I44" s="3" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>Texas A&amp;M University invites applications for multiple faculty positions in Computer Science and Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
-        </is>
-      </c>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t>http://engineering.academickeys.com/job/rh7lvag4/CSE--TAMU-Multiple-Faculty-Positions</t>
-        </is>
-      </c>
-      <c r="M44" s="3" t="inlineStr">
-        <is>
-          <t>AcademicKeys</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P44" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q44" s="2" t="n">
-        <v>30.6187</v>
-      </c>
-      <c r="R44" s="2" t="n">
-        <v>-96.3365</v>
-      </c>
-      <c r="S44" s="2" t="inlineStr">
-        <is>
-          <t>7d5d844d65485b4b</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Assistant Professor of Civil Engineering</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>McNeese State University</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>Moderate fit: broad Civil Engineering search where transportation is not explicitly prioritized in the snippet.</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>Civil Engineering, Engineering Education</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>Lake Charles, LA</t>
-        </is>
-      </c>
-      <c r="I45" s="3" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>$76,000 per year</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr">
-        <is>
-          <t>Assistant Professor position in Civil and Environmental Engineering at McNeese State University with a salary of $76,000 per year. | Research Topics: Civil Engineering, Engineering Education</t>
-        </is>
-      </c>
-      <c r="L45" s="5" t="inlineStr">
-        <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545361&amp;Title=Assistant%20Professor%20of%20Civil%20Engineering</t>
-        </is>
-      </c>
-      <c r="M45" s="3" t="inlineStr">
-        <is>
-          <t>HigherEdJobs</t>
-        </is>
-      </c>
-      <c r="N45" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O45" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P45" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q45" s="2" t="n">
-        <v>30.1751363</v>
-      </c>
-      <c r="R45" s="2" t="n">
-        <v>-93.2112786</v>
-      </c>
-      <c r="S45" s="2" t="inlineStr">
-        <is>
-          <t>bd292fb9f52ac2e9</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="26" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Tenure-Track Faculty Positions in Transportation Engineering</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>National Taiwan University</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Department of Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D46" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>Core match: seeks multiple tenure-track faculty positions specifically in the Transportation track within a Department of Civil Engineering.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Transportation Engineering, Mobility Systems, Transit Planning</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>Tenure-Track</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>Taipei, Taiwan</t>
-        </is>
-      </c>
-      <c r="I46" s="3" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>NT$83,720–137,370 monthly</t>
-        </is>
-      </c>
-      <c r="K46" s="4" t="inlineStr">
-        <is>
-          <t>The Department of Civil Engineering at National Taiwan University invites applications for multiple tenure-track faculty positions in Transportation Engineering. | Research Topics: Transportation Engineering, Mobility Systems, Transit Planning</t>
-        </is>
-      </c>
-      <c r="L46" s="5" t="inlineStr">
-        <is>
-          <t>https://jobs.chronicle.com/job/38034402/faculty-recruitment-announcement-department-of-civil-engineering-national-taiwan-university/</t>
-        </is>
-      </c>
-      <c r="M46" s="3" t="inlineStr">
-        <is>
-          <t>Chronicle</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P46" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="n">
-        <v>25.0375198</v>
-      </c>
-      <c r="R46" s="2" t="n">
-        <v>121.5636796</v>
-      </c>
-      <c r="S46" s="2" t="inlineStr">
-        <is>
-          <t>f056997ace2e1de7</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="26" customHeight="1">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Assistant Professor of Public Policy and Administration</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>University of Texas at Arlington</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Department of Public Affairs &amp; Planning</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>Moderate fit: Assistant Professor in Public Affairs &amp; Planning focused on public policy and urban studies, offering potential interdisciplinary overlap despite lacking a specific transportation mandate.</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>Tenure-Track</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>Arlington, TX</t>
-        </is>
-      </c>
-      <c r="I47" s="3" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr">
-        <is>
-          <t>The University of Texas at Arlington seeks a tenure-track Assistant Professor in Public Policy &amp; Planning to conduct policy research, secure external funding, and teach public administration courses requiring a Ph.D. | Research Topics: Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
-        </is>
-      </c>
-      <c r="L47" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-at-excel-campus-activities-4464851831</t>
-        </is>
-      </c>
-      <c r="M47" s="3" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="N47" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O47" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P47" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q47" s="2" t="n">
-        <v>32.7315155</v>
-      </c>
-      <c r="R47" s="2" t="n">
-        <v>-97.1171533</v>
-      </c>
-      <c r="S47" s="2" t="inlineStr">
         <is>
           <t>15704bb25858281c</t>
         </is>
@@ -4844,10 +4480,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix City Colleges of Chicago coordinates to Chicago, IL and resolve Chronicle Listed University placeholder
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -622,7 +622,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Chronicle Listed University</t>
+          <t>Embry-Riddle Aeronautical University</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -694,10 +694,10 @@
         </is>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>29.2108147</v>
+        <v>29.1895</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>-81.0228331</v>
+        <v>-81.04940000000001</v>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
@@ -785,10 +785,10 @@
         </is>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>32.898417</v>
+        <v>41.8837</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>-80.05262430000001</v>
+        <v>-87.6324</v>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Support full-page job text scraping, yearless deadline inference, and dual Priority/Final deadline handling
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S43"/>
+  <dimension ref="A1:S42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
     <col width="151" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="83" customWidth="1" min="9" max="9"/>
+    <col width="49" customWidth="1" min="9" max="9"/>
     <col width="96" customWidth="1" min="10" max="10"/>
     <col width="42" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -928,7 +928,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Priority: 2026-09-15 / Final: 2026-11-01</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -2801,30 +2801,30 @@
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Tenure-Track Assistant/Associate Professor of Air Transportation Systems</t>
+          <t>Assistant Professor / Associate Professor (Tenure-Track) in Civil and Environmental Engineering</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Embry-Riddle Aeronautical University</t>
+          <t>Nanyang Technological University</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>School of Graduate Studies in the College of Aviation</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>4</v>
+          <t>School of Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Moderate-low fit: the position focuses specifically on aviation and aerospace systems (air transportation, advanced air mobility, UAS) rather than surface transportation engineering or mobility.</t>
+          <t>Moderate fit: broad Civil and Environmental Engineering search where Transportation Engineering is a potential sub-discipline, though specific subfield requirements are not detailed in the snippet.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Air Transportation Systems, Advanced Air Mobility, UAS Traffic Management, Machine Learning/AI in Aviation</t>
+          <t>Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -2834,12 +2834,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Daytona Beach, FL</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Review begins immediately; Priority given to applications received by 2026-08-31</t>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2849,27 +2849,27 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>This tenure-track faculty position requires a doctorate in air transportation systems, advanced air mobility, or a related area to teach graduate courses and conduct AI/machine learning research in aviation. | Research Topics: Air Transportation Systems, Advanced Air Mobility, UAS Traffic Management, Machine Learning/AI in Aviation</t>
+          <t>Tenure-track Assistant or Associate Professor position in Civil and Environmental Engineering requiring an earned doctorate in civil engineering or a closely related discipline. | Research Topics: Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/tenure-track-faculty-position-with-a-focus-on-air-transportation-systems-daytona-beach-campus-at-embry-riddle-aeronautical-university-4434897662</t>
+          <t>https://engineering.academickeys.com/job/dhzin0q4/Assistant-Professor--Associate-Professor-TenureTrack-in-Civil-and-Environmental-Engineering</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P26" s="3" t="inlineStr">
@@ -2878,44 +2878,44 @@
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>33.8082375</v>
+        <v>1.2899175</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>-118.1344224</v>
+        <v>103.8519072</v>
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>b3c177958e0ab7a7</t>
+          <t>3fa57c30724444e8</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor / Associate Professor (Tenure-Track) in Civil and Environmental Engineering</t>
+          <t>Assistant / Associate / Full Professor of Mechanical Engineering</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Nanyang Technological University</t>
+          <t>Auburn University</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>School of Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>5</v>
+          <t>Department of Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: broad Civil and Environmental Engineering search where Transportation Engineering is a potential sub-discipline, though specific subfield requirements are not detailed in the snippet.</t>
+          <t>Low fit: position is in Mechanical Engineering and lacks description details, which does not align with the candidate's transportation engineering and planning profile.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
+          <t>Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -2925,12 +2925,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Singapore, Singapore</t>
+          <t>Auburn, AL</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2940,12 +2940,12 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Tenure-track Assistant or Associate Professor position in Civil and Environmental Engineering requiring an earned doctorate in civil engineering or a closely related discipline. | Research Topics: Civil and Environmental Engineering, Transportation Systems, Infrastructure Systems, Smart Cities</t>
+          <t>An open-rank faculty position in mechanical engineering requiring a Ph.D. in mechanical engineering or a closely related field. | Research Topics: Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>https://engineering.academickeys.com/job/dhzin0q4/Assistant-Professor--Associate-Professor-TenureTrack-in-Civil-and-Environmental-Engineering</t>
+          <t>https://engineering.academickeys.com/job/f320isty/AssistantAssociateFull-Professor</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
@@ -2969,44 +2969,44 @@
         </is>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>1.2899175</v>
+        <v>32.5919529</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>103.8519072</v>
+        <v>-85.4959775</v>
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>3fa57c30724444e8</t>
+          <t>c08698a4bf95171b</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Assistant / Associate / Full Professor of Mechanical Engineering</t>
+          <t>Assistant / Associate Professor of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Auburn University</t>
+          <t>University of Washington</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Department of Mechanical Engineering</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>3</v>
+          <t>Industrial and Systems Engineering</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>7</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Low fit: position is in Mechanical Engineering and lacks description details, which does not align with the candidate's transportation engineering and planning profile.</t>
+          <t>Strong interdisciplinary match: industrial and systems engineering position in a target department, though specific mobility focus depends on the full department scope.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
+          <t>Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -3016,27 +3016,27 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Auburn, AL</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>An open-rank faculty position in mechanical engineering requiring a Ph.D. in mechanical engineering or a closely related field. | Research Topics: Mechanical Engineering, Thermal/Fluids or Mechanical Systems</t>
+          <t>Assistant or Associate Professor position in Industrial and Systems Engineering requiring a Ph.D. in a relevant engineering or analytical discipline. | Research Topics: Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>https://engineering.academickeys.com/job/f320isty/AssistantAssociateFull-Professor</t>
+          <t>https://engineering.academickeys.com/job/g4m97a60/AssistantAssociate-Professor-Industrial-and-Systems-Engineering-Systems-Engineering-Focus</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
@@ -3060,59 +3060,59 @@
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>32.5919529</v>
+        <v>47.6553</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>-85.4959775</v>
+        <v>-122.3035</v>
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>c08698a4bf95171b</t>
+          <t>9d5682cf4dbca334</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Assistant / Associate Professor of Industrial and Systems Engineering</t>
+          <t>Professor &amp; Department Chair</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>University of Washington</t>
+          <t>University of Pittsburgh</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Industrial and Systems Engineering</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>7</v>
+          <t>Department of Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Strong interdisciplinary match: industrial and systems engineering position in a target department, though specific mobility focus depends on the full department scope.</t>
+          <t>Low fit: departmental leadership position for a broad Civil and Environmental Engineering department rather than a dedicated transportation research faculty role.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
+          <t>Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Tenured</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -3122,12 +3122,12 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Assistant or Associate Professor position in Industrial and Systems Engineering requiring a Ph.D. in a relevant engineering or analytical discipline. | Research Topics: Industrial and Systems Engineering, Mobility Systems, Systems Optimization</t>
+          <t>Strictly 1 concise sentence summarizing the primary focus of the role and minimum degree qualification. | Research Topics: Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>https://engineering.academickeys.com/job/g4m97a60/AssistantAssociate-Professor-Industrial-and-Systems-Engineering-Systems-Engineering-Focus</t>
+          <t>http://engineering.academickeys.com/job/vhlo0w6p/Professor--Department-Chair--Electrical-and-Computer-Engineering</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
@@ -3151,59 +3151,59 @@
         </is>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>47.6553</v>
+        <v>40.444153</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>-122.3035</v>
+        <v>-79.962461</v>
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>9d5682cf4dbca334</t>
+          <t>17acd4b4e7207871</t>
         </is>
       </c>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Professor &amp; Department Chair</t>
+          <t>Lecturer in Discipline or Senior Lecturer in Discipline</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>University of Pittsburgh</t>
+          <t>Columbia University</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>3</v>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Low fit: departmental leadership position for a broad Civil and Environmental Engineering department rather than a dedicated transportation research faculty role.</t>
+          <t>Moderate fit: general lecturer position at Columbia University in an unspecified discipline, requiring further text details to confirm a transportation focus.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
+          <t>Higher Education, Instruction, Academic Teaching</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Tenured</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3213,12 +3213,12 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>Strictly 1 concise sentence summarizing the primary focus of the role and minimum degree qualification. | Research Topics: Civil Engineering, Environmental Engineering, Academic Leadership, Departmental Administration</t>
+          <t>This is a faculty teaching role at Columbia University, though the specific academic department and subject focus are missing from the current snippet. | Research Topics: Higher Education, Instruction, Academic Teaching</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>http://engineering.academickeys.com/job/vhlo0w6p/Professor--Department-Chair--Electrical-and-Computer-Engineering</t>
+          <t>http://engineering.academickeys.com/job/arsy3jqh/Open-Rank-Lecturer-in-Discipline-or-Senior-Lecturer-in-Discipline</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -3242,79 +3242,79 @@
         </is>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>40.444153</v>
+        <v>40.8077507</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>-79.962461</v>
+        <v>-73.9624901</v>
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>17acd4b4e7207871</t>
+          <t>f11b4a4e74422ae3</t>
         </is>
       </c>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Lecturer in Discipline or Senior Lecturer in Discipline</t>
+          <t>Assistant/Associate Professor of Civil Engineering</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Columbia University</t>
+          <t>Cedarville University</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
+          <t>Department of Civil Engineering</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Moderate fit: broad Civil Engineering search where transportation may be acceptable, but lacks a dedicated job description snippet for precise evaluation.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Tenure-Track</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Cedarville, OH</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="D31" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Moderate fit: general lecturer position at Columbia University in an unspecified discipline, requiring further text details to confirm a transportation focus.</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Higher Education, Instruction, Academic Teaching</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Non-Tenure Track</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>New York, NY</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>This is a faculty teaching role at Columbia University, though the specific academic department and subject focus are missing from the current snippet. | Research Topics: Higher Education, Instruction, Academic Teaching</t>
+          <t>A faculty position in civil engineering requiring a Ph.D. to teach undergraduate courses and engage in scholarly activity. | Research Topics: Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>http://engineering.academickeys.com/job/arsy3jqh/Open-Rank-Lecturer-in-Discipline-or-Senior-Lecturer-in-Discipline</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179544290&amp;Title=Assistant%2FAssociate%20Professor%20of%20Civil%20Engineering</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>AcademicKeys</t>
+          <t>HigherEdJobs</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -3333,44 +3333,44 @@
         </is>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>40.8077507</v>
+        <v>39.7540491</v>
       </c>
       <c r="R31" s="2" t="n">
-        <v>-73.9624901</v>
+        <v>-83.8170518</v>
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>f11b4a4e74422ae3</t>
+          <t>751c7406865a2787</t>
         </is>
       </c>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate Professor of Civil Engineering</t>
+          <t>Professor, Associate Professor, or Assistant Professor of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Cedarville University</t>
+          <t>Auburn University</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil Engineering</t>
+          <t>Department of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="D32" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: broad Civil Engineering search where transportation may be acceptable, but lacks a dedicated job description snippet for precise evaluation.</t>
+          <t>Moderate fit: Industrial and Systems Engineering faculty position at Auburn University, but the job description text was missing to confirm a specific focus on mobility systems.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
+          <t>Industrial Engineering, Systems Engineering, Operations Research</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -3380,27 +3380,27 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Cedarville, OH</t>
+          <t>Auburn, AL</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Open until filled</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$80,000 - $180,000 per year</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>A faculty position in civil engineering requiring a Ph.D. to teach undergraduate courses and engage in scholarly activity. | Research Topics: Civil Engineering, Transportation Engineering, Infrastructure Systems</t>
+          <t>Open-rank faculty position in Industrial and Systems Engineering requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Systems Engineering, Operations Research</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179544290&amp;Title=Assistant%2FAssociate%20Professor%20of%20Civil%20Engineering</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179548357&amp;Title=Professor%2C%20Associate%20Professor%2C%20Assistant%20Professor%20%2D%20Industrial%20and%20Systems%20Engineering</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
@@ -3424,54 +3424,54 @@
         </is>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>39.7540491</v>
+        <v>32.5919529</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>-83.8170518</v>
+        <v>-85.4959775</v>
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>751c7406865a2787</t>
+          <t>d0f23a527bf71c22</t>
         </is>
       </c>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Professor, Associate Professor, or Assistant Professor of Industrial and Systems Engineering</t>
+          <t>Teaching Assistant Professor</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Auburn University</t>
+          <t>University of Arkansas</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial and Systems Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: Industrial and Systems Engineering faculty position at Auburn University, but the job description text was missing to confirm a specific focus on mobility systems.</t>
+          <t>Moderate fit: Broad Civil Engineering faculty search where transportation is only one of multiple acceptable sub-disciplines.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Industrial Engineering, Systems Engineering, Operations Research</t>
+          <t>Civil Engineering Education, Transportation Engineering</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Non-Tenure Track</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Auburn, AL</t>
+          <t>Fayetteville, AR</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>$80,000 - $180,000 per year</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Open-rank faculty position in Industrial and Systems Engineering requiring a Ph.D. in industrial engineering, systems engineering, or a closely related field. | Research Topics: Industrial Engineering, Systems Engineering, Operations Research</t>
+          <t>A teaching-focused assistant professor position in civil engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Civil Engineering Education, Transportation Engineering</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179548357&amp;Title=Professor%2C%20Associate%20Professor%2C%20Assistant%20Professor%20%2D%20Industrial%20and%20Systems%20Engineering</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179541925&amp;Title=Teaching%20Assistant%20Professor</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -3515,31 +3515,31 @@
         </is>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>32.5919529</v>
+        <v>36.0970389</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>-85.4959775</v>
+        <v>-94.1703322</v>
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>d0f23a527bf71c22</t>
+          <t>8b28f5b58e7e3607</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Teaching Assistant Professor</t>
+          <t>Assistant Professor of Teaching</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>Florida Atlantic University</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Department of Civil, Environmental &amp; Geomatics Engineering</t>
         </is>
       </c>
       <c r="D34" s="7" t="n">
@@ -3547,12 +3547,12 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: Broad Civil Engineering faculty search where transportation is only one of multiple acceptable sub-disciplines.</t>
+          <t>Moderate fit: it is a Civil Engineering teaching position in a department with transportation research centers, but requires teaching structural analysis and design-related classes alongside a P.E. license.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering Education, Transportation Engineering</t>
+          <t>Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -3562,7 +3562,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
+          <t>Boca Raton, FL</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -3572,22 +3572,22 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Commensurate with Experience</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>A teaching-focused assistant professor position in civil engineering requiring a Ph.D. in civil engineering or a closely related field. | Research Topics: Civil Engineering Education, Transportation Engineering</t>
+          <t>This is a non-tenure-track Assistant Teaching Professor position in civil engineering requiring a Ph.D. and P.E. license to teach undergraduate and graduate courses including structural analysis and design. | Research Topics: Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179541925&amp;Title=Teaching%20Assistant%20Professor</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-teaching-at-florida-atlantic-university-4414964381</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>HigherEdJobs</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">
@@ -3606,74 +3606,74 @@
         </is>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>36.0970389</v>
+        <v>26.1194058</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>-94.1703322</v>
+        <v>-80.14167999999999</v>
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>8b28f5b58e7e3607</t>
+          <t>7bdaa996cf64d1f6</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Teaching</t>
+          <t>Assistant or Associate Professor in Supply Chain Management</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Florida Atlantic University</t>
+          <t>University of Arkansas</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil, Environmental &amp; Geomatics Engineering</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="n">
-        <v>5</v>
+          <t>J.B. Hunt Transport Department of Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: it is a Civil Engineering teaching position in a department with transportation research centers, but requires teaching structural analysis and design-related classes alongside a P.E. license.</t>
+          <t>Low fit: this is a faculty position in Supply Chain Management within a Business School rather than Transportation Engineering.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+          <t>Supply Chain Management, Logistics, Operations Research</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Non-Tenure Track</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Boca Raton, FL</t>
+          <t>Fayetteville, AR</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Commensurate with Experience</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>This is a non-tenure-track Assistant Teaching Professor position in civil engineering requiring a Ph.D. and P.E. license to teach undergraduate and graduate courses including structural analysis and design. | Research Topics: Civil Engineering Education, Applied Transportation Problems, Infrastructure and Sustainability</t>
+          <t>This is a tenure-track Assistant or Associate Professor position in Supply Chain Management requiring a strong research record in leading peer-reviewed journals. | Research Topics: Supply Chain Management, Logistics, Operations Research</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-of-teaching-at-florida-atlantic-university-4414964381</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-or-associate-professor-open-rank-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460111187</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P35" s="3" t="inlineStr">
@@ -3697,31 +3697,31 @@
         </is>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>26.1194058</v>
+        <v>36.0625843</v>
       </c>
       <c r="R35" s="2" t="n">
-        <v>-80.14167999999999</v>
+        <v>-94.1574328</v>
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>7bdaa996cf64d1f6</t>
+          <t>c16a694d5f7f68d4</t>
         </is>
       </c>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Assistant or Associate Professor in Supply Chain Management</t>
+          <t>Assistant Professor of Aerospace Engineering</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>The University of Kansas</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>J.B. Hunt Transport Department of Supply Chain Management</t>
+          <t>Department of Aerospace Engineering</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -3729,12 +3729,12 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Low fit: this is a faculty position in Supply Chain Management within a Business School rather than Transportation Engineering.</t>
+          <t>The position is specifically for Aerospace Engineering focusing on aircraft and space systems, where the candidate's core transportation engineering expertise is not the primary requirement.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Logistics, Operations Research</t>
+          <t>Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -3744,12 +3744,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Fayetteville, AR</t>
+          <t>Lawrence, KS</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3759,12 +3759,12 @@
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track Assistant or Associate Professor position in Supply Chain Management requiring a strong research record in leading peer-reviewed journals. | Research Topics: Supply Chain Management, Logistics, Operations Research</t>
+          <t>This is a tenure-track faculty position in Aerospace Engineering requiring a doctorate in Aerospace Engineering or a closely related field, focusing on aviation and space-related research. | Research Topics: Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-or-associate-professor-open-rank-at-university-of-arkansas-%C2%AD-sam-m-walton-college-of-business-4460111187</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-aerospace-engineering-at-the-university-of-kansas-4460398978</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
@@ -3788,44 +3788,44 @@
         </is>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>36.0625843</v>
+        <v>39.0559267</v>
       </c>
       <c r="R36" s="2" t="n">
-        <v>-94.1574328</v>
+        <v>-94.6090332</v>
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>c16a694d5f7f68d4</t>
+          <t>4a53cfad86712a72</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Aerospace Engineering</t>
+          <t>Assistant/Associate/Full Professor in Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>The University of Kansas</t>
+          <t>University of Florida</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Department of Aerospace Engineering</t>
+          <t>Department of Industrial and Systems Engineering</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>The position is specifically for Aerospace Engineering focusing on aircraft and space systems, where the candidate's core transportation engineering expertise is not the primary requirement.</t>
+          <t>Moderate fit: while housed in Industrial and Systems Engineering with a broad mention of transportation applications, the primary departmental focus and hiring emphasis is strictly on Industrialized Construction.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+          <t>Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -3835,27 +3835,27 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Lawrence, KS</t>
+          <t>Gainesville, FL</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>This is a tenure-track faculty position in Aerospace Engineering requiring a doctorate in Aerospace Engineering or a closely related field, focusing on aviation and space-related research. | Research Topics: Unmanned aircraft, Advanced air mobility, Aerospace autonomy, Space systems engineering</t>
+          <t>The Department of Industrial and Systems Engineering at the University of Florida seeks a tenured/tenure-track faculty member specializing in Industrialized Construction with a PhD in ISE, Manufacturing Engineering, Civil Engineering, Mechanical Engineering, or a closely related field. | Research Topics: Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-aerospace-engineering-at-the-university-of-kansas-4460398978</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-industrial-systems-engineering-at-university-of-florida-4323668785</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="P37" s="3" t="inlineStr">
@@ -3879,44 +3879,44 @@
         </is>
       </c>
       <c r="Q37" s="2" t="n">
-        <v>39.0559267</v>
+        <v>29.6436</v>
       </c>
       <c r="R37" s="2" t="n">
-        <v>-94.6090332</v>
+        <v>-82.3549</v>
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>4a53cfad86712a72</t>
+          <t>56d501f448e77e05</t>
         </is>
       </c>
     </row>
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Assistant/Associate/Full Professor in Industrial and Systems Engineering</t>
+          <t>Assistant Professor in Supply Chain Management</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>University of Florida</t>
+          <t>Iowa State University</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial and Systems Engineering</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="n">
-        <v>4</v>
+          <t>Department of Supply Chain Management, Ivy College of Business</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: while housed in Industrial and Systems Engineering with a broad mention of transportation applications, the primary departmental focus and hiring emphasis is strictly on Industrialized Construction.</t>
+          <t>Moderate fit: the role is in a business school supply chain department rather than engineering or planning, though it accepts transportation as a related specialization.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+          <t>Supply Chain Management, Transportation, Logistics, Operations</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Gainesville, FL</t>
+          <t>Ames, IA</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -3941,12 +3941,12 @@
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>The Department of Industrial and Systems Engineering at the University of Florida seeks a tenured/tenure-track faculty member specializing in Industrialized Construction with a PhD in ISE, Manufacturing Engineering, Civil Engineering, Mechanical Engineering, or a closely related field. | Research Topics: Industrialized Construction, Operations Research, Artificial Intelligence, Digital Twins</t>
+          <t>The Ivy College of Business at Iowa State University seeks a tenure-track Assistant Professor in Supply Chain Management to conduct research and teach across undergraduate, master's, and Ph.D. levels, requiring a Ph.D. in business administration or a related field such as transportation or logistics. | Research Topics: Supply Chain Management, Transportation, Logistics, Operations</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-associate-full-professor-industrial-systems-engineering-at-university-of-florida-4323668785</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-in-supply-chain-management-at-iowa-state-university-ivy-college-of-business-4440811209</t>
         </is>
       </c>
       <c r="M38" s="3" t="inlineStr">
@@ -3970,54 +3970,54 @@
         </is>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>29.6436</v>
+        <v>42.0267567</v>
       </c>
       <c r="R38" s="2" t="n">
-        <v>-82.3549</v>
+        <v>-93.6170448</v>
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>56d501f448e77e05</t>
+          <t>e994e392d38b77ce</t>
         </is>
       </c>
     </row>
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor in Supply Chain Management</t>
+          <t>Multiple Faculty Positions in Computer Science and Engineering</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Iowa State University</t>
+          <t>Texas A&amp;M University</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Department of Supply Chain Management, Ivy College of Business</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="n">
-        <v>6</v>
+          <t>Department of Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: the role is in a business school supply chain department rather than engineering or planning, though it accepts transportation as a related specialization.</t>
+          <t>Moderate fit: open faculty search in Computer Science and Engineering without explicit specialization in transportation or mobility systems.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Management, Transportation, Logistics, Operations</t>
+          <t>Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Tenure-Track</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Ames, IA</t>
+          <t>College Station, TX</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -4032,27 +4032,27 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>The Ivy College of Business at Iowa State University seeks a tenure-track Assistant Professor in Supply Chain Management to conduct research and teach across undergraduate, master's, and Ph.D. levels, requiring a Ph.D. in business administration or a related field such as transportation or logistics. | Research Topics: Supply Chain Management, Transportation, Logistics, Operations</t>
+          <t>Texas A&amp;M University invites applications for multiple faculty positions in Computer Science and Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
         </is>
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-in-supply-chain-management-at-iowa-state-university-ivy-college-of-business-4440811209</t>
+          <t>http://engineering.academickeys.com/job/rh7lvag4/CSE--TAMU-Multiple-Faculty-Positions</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>AcademicKeys</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="P39" s="3" t="inlineStr">
@@ -4061,44 +4061,44 @@
         </is>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>42.0267567</v>
+        <v>30.6187</v>
       </c>
       <c r="R39" s="2" t="n">
-        <v>-93.6170448</v>
+        <v>-96.3365</v>
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>e994e392d38b77ce</t>
+          <t>7d5d844d65485b4b</t>
         </is>
       </c>
     </row>
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Multiple Faculty Positions in Computer Science and Engineering</t>
+          <t>Assistant Professor of Civil Engineering</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Texas A&amp;M University</t>
+          <t>McNeese State University</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Department of Computer Science and Engineering</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>4</v>
+          <t>Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: open faculty search in Computer Science and Engineering without explicit specialization in transportation or mobility systems.</t>
+          <t>Moderate fit: broad Civil Engineering search where transportation is not explicitly prioritized in the snippet.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
+          <t>Civil Engineering, Engineering Education</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>College Station, TX</t>
+          <t>Lake Charles, LA</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -4118,22 +4118,22 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>$76,000 per year</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>Texas A&amp;M University invites applications for multiple faculty positions in Computer Science and Engineering, requiring a Ph.D. in a relevant discipline. | Research Topics: Computer Science, Computer Engineering, Artificial Intelligence, Data Science</t>
+          <t>Assistant Professor position in Civil and Environmental Engineering at McNeese State University with a salary of $76,000 per year. | Research Topics: Civil Engineering, Engineering Education</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>http://engineering.academickeys.com/job/rh7lvag4/CSE--TAMU-Multiple-Faculty-Positions</t>
+          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545361&amp;Title=Assistant%20Professor%20of%20Civil%20Engineering</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t>AcademicKeys</t>
+          <t>HigherEdJobs</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -4152,79 +4152,79 @@
         </is>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>30.6187</v>
+        <v>30.1751363</v>
       </c>
       <c r="R40" s="2" t="n">
-        <v>-96.3365</v>
+        <v>-93.2112786</v>
       </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
-          <t>7d5d844d65485b4b</t>
+          <t>bd292fb9f52ac2e9</t>
         </is>
       </c>
     </row>
     <row r="41" ht="26" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Civil Engineering</t>
+          <t>Tenure-Track Faculty Positions in Transportation Engineering</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>McNeese State University</t>
+          <t>National Taiwan University</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Civil and Environmental Engineering</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="n">
-        <v>5</v>
+          <t>Department of Civil Engineering</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>9</v>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Moderate fit: broad Civil Engineering search where transportation is not explicitly prioritized in the snippet.</t>
+          <t>Core match: seeks multiple tenure-track faculty positions specifically in the Transportation track within a Department of Civil Engineering.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering, Engineering Education</t>
+          <t>Transportation Engineering, Mobility Systems, Transit Planning</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Tenure-Track</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Lake Charles, LA</t>
+          <t>Taipei, Taiwan</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Open until filled</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>$76,000 per year</t>
+          <t>NT$83,720–137,370 monthly</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Assistant Professor position in Civil and Environmental Engineering at McNeese State University with a salary of $76,000 per year. | Research Topics: Civil Engineering, Engineering Education</t>
+          <t>The Department of Civil Engineering at National Taiwan University invites applications for multiple tenure-track faculty positions in Transportation Engineering. | Research Topics: Transportation Engineering, Mobility Systems, Transit Planning</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>https://www.higheredjobs.com/search/details.cfm?JobCode=179545361&amp;Title=Assistant%20Professor%20of%20Civil%20Engineering</t>
+          <t>https://jobs.chronicle.com/job/38034402/faculty-recruitment-announcement-department-of-civil-engineering-national-taiwan-university/</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>HigherEdJobs</t>
+          <t>Chronicle</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -4243,44 +4243,44 @@
         </is>
       </c>
       <c r="Q41" s="2" t="n">
-        <v>30.1751363</v>
+        <v>25.0375198</v>
       </c>
       <c r="R41" s="2" t="n">
-        <v>-93.2112786</v>
+        <v>121.5636796</v>
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>bd292fb9f52ac2e9</t>
+          <t>f056997ace2e1de7</t>
         </is>
       </c>
     </row>
     <row r="42" ht="26" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Tenure-Track Faculty Positions in Transportation Engineering</t>
+          <t>Assistant Professor of Public Policy and Administration</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>National Taiwan University</t>
+          <t>University of Texas at Arlington</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Department of Civil Engineering</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="n">
-        <v>9</v>
+          <t>Department of Public Affairs &amp; Planning</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Core match: seeks multiple tenure-track faculty positions specifically in the Transportation track within a Department of Civil Engineering.</t>
+          <t>Moderate fit: Assistant Professor in Public Affairs &amp; Planning focused on public policy and urban studies, offering potential interdisciplinary overlap despite lacking a specific transportation mandate.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Transportation Engineering, Mobility Systems, Transit Planning</t>
+          <t>Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -4290,32 +4290,32 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Taipei, Taiwan</t>
+          <t>Arlington, TX</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
+          <t>Open until filled</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>NT$83,720–137,370 monthly</t>
-        </is>
-      </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>The Department of Civil Engineering at National Taiwan University invites applications for multiple tenure-track faculty positions in Transportation Engineering. | Research Topics: Transportation Engineering, Mobility Systems, Transit Planning</t>
+          <t>The University of Texas at Arlington seeks a tenure-track Assistant Professor in Public Policy &amp; Planning to conduct policy research, secure external funding, and teach public administration courses requiring a Ph.D. | Research Topics: Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
         </is>
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.chronicle.com/job/38034402/faculty-recruitment-announcement-department-of-civil-engineering-national-taiwan-university/</t>
+          <t>https://www.linkedin.com/jobs/view/assistant-professor-at-excel-campus-activities-4464851831</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>Chronicle</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -4334,103 +4334,12 @@
         </is>
       </c>
       <c r="Q42" s="2" t="n">
-        <v>25.0375198</v>
+        <v>32.7315155</v>
       </c>
       <c r="R42" s="2" t="n">
-        <v>121.5636796</v>
+        <v>-97.1171533</v>
       </c>
       <c r="S42" s="2" t="inlineStr">
-        <is>
-          <t>f056997ace2e1de7</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Assistant Professor of Public Policy and Administration</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>University of Texas at Arlington</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Department of Public Affairs &amp; Planning</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>Moderate fit: Assistant Professor in Public Affairs &amp; Planning focused on public policy and urban studies, offering potential interdisciplinary overlap despite lacking a specific transportation mandate.</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Tenure-Track</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Arlington, TX</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>Open until filled</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr">
-        <is>
-          <t>The University of Texas at Arlington seeks a tenure-track Assistant Professor in Public Policy &amp; Planning to conduct policy research, secure external funding, and teach public administration courses requiring a Ph.D. | Research Topics: Public Policy, Urban Studies, Public Infrastructure, Interdisciplinary Public Administration</t>
-        </is>
-      </c>
-      <c r="L43" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/assistant-professor-at-excel-campus-activities-4464851831</t>
-        </is>
-      </c>
-      <c r="M43" s="3" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="N43" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O43" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="P43" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="Q43" s="2" t="n">
-        <v>32.7315155</v>
-      </c>
-      <c r="R43" s="2" t="n">
-        <v>-97.1171533</v>
-      </c>
-      <c r="S43" s="2" t="inlineStr">
         <is>
           <t>15704bb25858281c</t>
         </is>
@@ -4479,7 +4388,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>